<commit_message>
Fix yearly/monthly return calculation + quality check (60/60 PASS)
Bug fixed: yearly returns used first-trading-day NAV (missing day 1 return).
Now uses year-end NAV ratios matching monthly compound exactly.
Monthly returns also fixed to use month-end NAV ratios.

Quality check (60 tests):
- All CAGR, MaxDD, Worst5Y, Worst10Y match across CSV/recalculation
- Monthly compound == yearly return for all years (diff=0.00%)
- DD transitions = 34, BH trades = 0
- A2 2001-2002 = 0% (CASH confirmed)
- BH 3x MaxDD = -99.89% (confirmed)

https://claude.ai/code/session_01AnaE6CMbDeeFYPv77Xs27G
</commit_message>
<xml_diff>
--- a/YEARLY_RETURNS_7STRATEGIES.xlsx
+++ b/YEARLY_RETURNS_7STRATEGIES.xlsx
@@ -807,25 +807,25 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>0.1646020169450002</v>
+        <v>0.1665996899649919</v>
       </c>
       <c r="C17" s="12" t="n">
-        <v>0.2881129415652957</v>
+        <v>0.2724172919543411</v>
       </c>
       <c r="D17" s="12" t="n">
-        <v>0.2875823048216108</v>
+        <v>0.2618094703587007</v>
       </c>
       <c r="E17" s="12" t="n">
-        <v>0.1504599219668634</v>
+        <v>0.1902055975229084</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>0.2167586779061725</v>
+        <v>0.240454275842977</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>0.3943631388173681</v>
+        <v>0.4441473437933345</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>0.1492147038401792</v>
+        <v>0.1545348787862986</v>
       </c>
     </row>
     <row r="18">
@@ -835,25 +835,25 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>0.5612180864346796</v>
+        <v>0.5661043833464285</v>
       </c>
       <c r="C18" s="12" t="n">
-        <v>1.322614638780552</v>
+        <v>1.35875267377596</v>
       </c>
       <c r="D18" s="12" t="n">
-        <v>2.147581131823013</v>
+        <v>2.213621488235486</v>
       </c>
       <c r="E18" s="12" t="n">
-        <v>1.421624751140155</v>
+        <v>1.472433596080058</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>3.947844227873866</v>
+        <v>4.051656451482201</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>3.947844227873868</v>
+        <v>4.051656451482202</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>0.8429428539642675</v>
+        <v>0.8558529333810629</v>
       </c>
     </row>
     <row r="19">
@@ -863,25 +863,25 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>-0.1137437203285541</v>
+        <v>-0.1106437953990623</v>
       </c>
       <c r="C19" s="12" t="n">
-        <v>-0.1491924803278044</v>
+        <v>-0.1265113932269826</v>
       </c>
       <c r="D19" s="12" t="n">
-        <v>-0.2765712428625557</v>
+        <v>-0.2507263406918773</v>
       </c>
       <c r="E19" s="12" t="n">
         <v>-0.4275134999314306</v>
       </c>
       <c r="F19" s="12" t="n">
-        <v>-0.479103160634812</v>
+        <v>-0.4636589594432232</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>-0.8969672477188233</v>
+        <v>-0.8922735087553108</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>-0.4019776385253038</v>
+        <v>-0.4054059104782409</v>
       </c>
     </row>
     <row r="20">
@@ -891,25 +891,25 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>0.1675255685775595</v>
+        <v>0.1670985173453593</v>
       </c>
       <c r="C20" s="12" t="n">
-        <v>0.2942030456680421</v>
+        <v>0.2943119212659813</v>
       </c>
       <c r="D20" s="12" t="n">
-        <v>0.4421676034697816</v>
+        <v>0.4445165596702268</v>
       </c>
       <c r="E20" s="12" t="n">
-        <v>0.3999629459013726</v>
+        <v>0.4004816133786941</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>0.7422752240329448</v>
+        <v>0.7519632177887554</v>
       </c>
       <c r="G20" s="12" t="n">
-        <v>0.8894134771351301</v>
+        <v>0.9059580471250496</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>0.2490738946141068</v>
+        <v>0.2525553450451991</v>
       </c>
     </row>
     <row r="21">
@@ -925,16 +925,16 @@
         <v>44</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F21" s="13" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H21" s="13" t="n">
         <v>39</v>
@@ -953,16 +953,16 @@
         <v>9</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H22" s="13" t="n">
         <v>14</v>
@@ -1048,10 +1048,10 @@
         <v>1975</v>
       </c>
       <c r="B27" s="16" t="n">
-        <v>-0.000188950536929799</v>
+        <v>-0.0008052275150162149</v>
       </c>
       <c r="C27" s="15" t="n">
-        <v>0.052544349967244</v>
+        <v>0.05206122966712612</v>
       </c>
       <c r="D27" s="15" t="n">
         <v>0.1440942281560682</v>
@@ -1063,10 +1063,10 @@
         <v>0.03829465497279538</v>
       </c>
       <c r="G27" s="15" t="n">
-        <v>0.9684960040191332</v>
+        <v>1.055303371427614</v>
       </c>
       <c r="H27" s="15" t="n">
-        <v>0.2787479690486332</v>
+        <v>0.2975593948512203</v>
       </c>
     </row>
     <row r="28">
@@ -1074,25 +1074,25 @@
         <v>1976</v>
       </c>
       <c r="B28" s="15" t="n">
-        <v>0.2887696395007184</v>
+        <v>0.2933320755275626</v>
       </c>
       <c r="C28" s="15" t="n">
-        <v>0.497004630931378</v>
+        <v>0.5082880300514738</v>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.6626211746295709</v>
+        <v>0.6825772668916013</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>0.3429764990045236</v>
+        <v>0.3515468080259636</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>0.912513841844483</v>
+        <v>0.9449722721229983</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>0.912513841844482</v>
+        <v>0.9449722721229972</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>0.2539072445274724</v>
+        <v>0.2610151148796012</v>
       </c>
     </row>
     <row r="29">
@@ -1100,25 +1100,25 @@
         <v>1977</v>
       </c>
       <c r="B29" s="15" t="n">
-        <v>0.1021764519164734</v>
+        <v>0.09964894718738648</v>
       </c>
       <c r="C29" s="15" t="n">
-        <v>0.07425108564519634</v>
+        <v>0.06948039762331115</v>
       </c>
       <c r="D29" s="15" t="n">
-        <v>0.03184426748183977</v>
+        <v>0.02580031066730371</v>
       </c>
       <c r="E29" s="15" t="n">
-        <v>0.06903878605558589</v>
+        <v>0.06421800018873047</v>
       </c>
       <c r="F29" s="15" t="n">
-        <v>0.2167586779061725</v>
+        <v>0.2096315976531375</v>
       </c>
       <c r="G29" s="15" t="n">
-        <v>0.2167586779061721</v>
+        <v>0.2096315976531373</v>
       </c>
       <c r="H29" s="15" t="n">
-        <v>0.07534037106478908</v>
+        <v>0.07325302635634534</v>
       </c>
     </row>
     <row r="30">
@@ -1126,25 +1126,25 @@
         <v>1978</v>
       </c>
       <c r="B30" s="15" t="n">
-        <v>0.3093057511743429</v>
+        <v>0.2975583012728265</v>
       </c>
       <c r="C30" s="15" t="n">
-        <v>0.6772449413312809</v>
+        <v>0.643696279585937</v>
       </c>
       <c r="D30" s="15" t="n">
-        <v>0.6564384732319815</v>
+        <v>0.6105822073840994</v>
       </c>
       <c r="E30" s="15" t="n">
-        <v>0.5214301484531498</v>
+        <v>0.4822725675980139</v>
       </c>
       <c r="F30" s="15" t="n">
-        <v>0.1777210332053192</v>
+        <v>0.1423659268294953</v>
       </c>
       <c r="G30" s="15" t="n">
-        <v>0.3902344097789951</v>
+        <v>0.3484996661009494</v>
       </c>
       <c r="H30" s="15" t="n">
-        <v>0.1344231057692307</v>
+        <v>0.1230842420823157</v>
       </c>
     </row>
     <row r="31">
@@ -1152,10 +1152,10 @@
         <v>1979</v>
       </c>
       <c r="B31" s="15" t="n">
-        <v>0.5529109703607988</v>
+        <v>0.5571043007201588</v>
       </c>
       <c r="C31" s="15" t="n">
-        <v>0.4580260611336564</v>
+        <v>0.4623950050341969</v>
       </c>
       <c r="D31" s="15" t="n">
         <v>0.2066930732204824</v>
@@ -1167,10 +1167,10 @@
         <v>0.5457980743804514</v>
       </c>
       <c r="G31" s="15" t="n">
-        <v>1.018616308497662</v>
+        <v>1.011360936595652</v>
       </c>
       <c r="H31" s="15" t="n">
-        <v>0.2825865930952678</v>
+        <v>0.2810645461672008</v>
       </c>
     </row>
     <row r="32">
@@ -1178,25 +1178,25 @@
         <v>1980</v>
       </c>
       <c r="B32" s="15" t="n">
-        <v>0.2260686788882161</v>
+        <v>0.2017036379309736</v>
       </c>
       <c r="C32" s="15" t="n">
-        <v>0.6313523896002171</v>
+        <v>0.5648183306317341</v>
       </c>
       <c r="D32" s="15" t="n">
-        <v>0.8752444018468539</v>
+        <v>0.7724834783120376</v>
       </c>
       <c r="E32" s="15" t="n">
-        <v>0.6956834071166149</v>
+        <v>0.6245723151604474</v>
       </c>
       <c r="F32" s="15" t="n">
-        <v>0.5734326974214214</v>
+        <v>0.4806220196524136</v>
       </c>
       <c r="G32" s="15" t="n">
-        <v>1.335278646626797</v>
+        <v>1.197529638151174</v>
       </c>
       <c r="H32" s="15" t="n">
-        <v>0.3655935663844716</v>
+        <v>0.338758749098576</v>
       </c>
     </row>
     <row r="33">
@@ -1204,25 +1204,25 @@
         <v>1981</v>
       </c>
       <c r="B33" s="16" t="n">
-        <v>-0.1137437203285541</v>
+        <v>-0.1106437953990623</v>
       </c>
       <c r="C33" s="16" t="n">
-        <v>-0.1023337529613945</v>
+        <v>-0.09593607940668493</v>
       </c>
       <c r="D33" s="16" t="n">
-        <v>-0.08283139966101549</v>
+        <v>-0.07309568724104054</v>
       </c>
       <c r="E33" s="16" t="n">
-        <v>-0.2024150543003272</v>
+        <v>-0.1881334360696377</v>
       </c>
       <c r="F33" s="16" t="n">
-        <v>-0.3308044024169734</v>
+        <v>-0.31882173386503</v>
       </c>
       <c r="G33" s="16" t="n">
-        <v>-0.1556143847012096</v>
+        <v>-0.1404947500313195</v>
       </c>
       <c r="H33" s="16" t="n">
-        <v>-0.03787770516515277</v>
+        <v>-0.0321241481096004</v>
       </c>
     </row>
     <row r="34">
@@ -1230,10 +1230,10 @@
         <v>1982</v>
       </c>
       <c r="B34" s="15" t="n">
-        <v>0.5612180864346796</v>
+        <v>0.5512191972643201</v>
       </c>
       <c r="C34" s="15" t="n">
-        <v>0.6620769946727409</v>
+        <v>0.6545944354376791</v>
       </c>
       <c r="D34" s="15" t="n">
         <v>0.8239838912198256</v>
@@ -1245,10 +1245,10 @@
         <v>0.8783700771542569</v>
       </c>
       <c r="G34" s="15" t="n">
-        <v>0.582016352708818</v>
+        <v>0.5744497968815379</v>
       </c>
       <c r="H34" s="15" t="n">
-        <v>0.1886155842510897</v>
+        <v>0.1867341132911375</v>
       </c>
     </row>
     <row r="35">
@@ -1256,25 +1256,25 @@
         <v>1983</v>
       </c>
       <c r="B35" s="15" t="n">
-        <v>0.1942870035578388</v>
+        <v>0.1885935722942893</v>
       </c>
       <c r="C35" s="15" t="n">
-        <v>0.4355687301890323</v>
+        <v>0.4151055239708994</v>
       </c>
       <c r="D35" s="15" t="n">
-        <v>0.7607437206973391</v>
+        <v>0.7252954023677592</v>
       </c>
       <c r="E35" s="15" t="n">
-        <v>0.8056543726854971</v>
+        <v>0.7672532261801166</v>
       </c>
       <c r="F35" s="15" t="n">
-        <v>0.5478362263264407</v>
+        <v>0.511419981811658</v>
       </c>
       <c r="G35" s="15" t="n">
-        <v>0.6757316735719108</v>
+        <v>0.6363064079475294</v>
       </c>
       <c r="H35" s="15" t="n">
-        <v>0.2082050862258569</v>
+        <v>0.1987436048579048</v>
       </c>
     </row>
     <row r="36">
@@ -1282,10 +1282,10 @@
         <v>1984</v>
       </c>
       <c r="B36" s="16" t="n">
-        <v>-0.020844051266665</v>
+        <v>-0.02176933314168294</v>
       </c>
       <c r="C36" s="16" t="n">
-        <v>-0.02231878415960142</v>
+        <v>-0.02294568495468274</v>
       </c>
       <c r="D36" s="16" t="n">
         <v>-0.04681722901282615</v>
@@ -1297,10 +1297,10 @@
         <v>-0.04741847573568513</v>
       </c>
       <c r="G36" s="16" t="n">
-        <v>-0.3362010440892905</v>
+        <v>-0.3431571394391051</v>
       </c>
       <c r="H36" s="16" t="n">
-        <v>-0.1099664965967926</v>
+        <v>-0.1130653241981625</v>
       </c>
     </row>
     <row r="37">
@@ -1308,25 +1308,25 @@
         <v>1985</v>
       </c>
       <c r="B37" s="15" t="n">
-        <v>0.4579969672412212</v>
+        <v>0.4463036498993587</v>
       </c>
       <c r="C37" s="15" t="n">
-        <v>0.6801532977898914</v>
+        <v>0.6646476312475865</v>
       </c>
       <c r="D37" s="15" t="n">
-        <v>0.8441150841661438</v>
+        <v>0.8240836545452386</v>
       </c>
       <c r="E37" s="15" t="n">
-        <v>0.7195965625220129</v>
+        <v>0.6944848249424243</v>
       </c>
       <c r="F37" s="15" t="n">
-        <v>1.24297543584882</v>
+        <v>1.210220653843504</v>
       </c>
       <c r="G37" s="15" t="n">
-        <v>1.242975435848823</v>
+        <v>1.210220653843507</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>0.3212688162977342</v>
+        <v>0.3148522303152028</v>
       </c>
     </row>
     <row r="38">
@@ -1334,25 +1334,25 @@
         <v>1986</v>
       </c>
       <c r="B38" s="15" t="n">
-        <v>0.2612121749964467</v>
+        <v>0.2611171370865586</v>
       </c>
       <c r="C38" s="15" t="n">
-        <v>0.3480443609628858</v>
+        <v>0.3487203422238021</v>
       </c>
       <c r="D38" s="15" t="n">
-        <v>0.2875823048216108</v>
+        <v>0.2886556068116617</v>
       </c>
       <c r="E38" s="15" t="n">
-        <v>0.3437185199953711</v>
+        <v>0.3449134747241704</v>
       </c>
       <c r="F38" s="15" t="n">
-        <v>0.1870320107629993</v>
+        <v>0.1880876258292425</v>
       </c>
       <c r="G38" s="15" t="n">
-        <v>0.1870320107630012</v>
+        <v>0.1880876258292445</v>
       </c>
       <c r="H38" s="15" t="n">
-        <v>0.07323073230769239</v>
+        <v>0.07356107861300852</v>
       </c>
     </row>
     <row r="39">
@@ -1360,25 +1360,25 @@
         <v>1987</v>
       </c>
       <c r="B39" s="15" t="n">
-        <v>0.1090376337000112</v>
+        <v>0.1182046633499157</v>
       </c>
       <c r="C39" s="15" t="n">
-        <v>0.2079477993376007</v>
+        <v>0.2231196878436484</v>
       </c>
       <c r="D39" s="15" t="n">
-        <v>0.1107767757314209</v>
+        <v>0.1323394141692327</v>
       </c>
       <c r="E39" s="15" t="n">
-        <v>0.02969248894599641</v>
+        <v>0.041372327125347</v>
       </c>
       <c r="F39" s="16" t="n">
-        <v>-0.2959268887578508</v>
+        <v>-0.2693058017374666</v>
       </c>
       <c r="G39" s="16" t="n">
-        <v>-0.3438731103649714</v>
+        <v>-0.3190648756142185</v>
       </c>
       <c r="H39" s="16" t="n">
-        <v>-0.06426956746536006</v>
+        <v>-0.05246556373161337</v>
       </c>
     </row>
     <row r="40">
@@ -1386,10 +1386,10 @@
         <v>1988</v>
       </c>
       <c r="B40" s="16" t="n">
-        <v>-0.03502642170219961</v>
+        <v>-0.03709610666342189</v>
       </c>
       <c r="C40" s="16" t="n">
-        <v>-0.05314771531352425</v>
+        <v>-0.05509604365913301</v>
       </c>
       <c r="D40" s="16" t="n">
         <v>-0.04009659602281069</v>
@@ -1401,10 +1401,10 @@
         <v>-0.05901039116474072</v>
       </c>
       <c r="G40" s="15" t="n">
-        <v>0.3783054416815745</v>
+        <v>0.4783471504169352</v>
       </c>
       <c r="H40" s="15" t="n">
-        <v>0.1267355805022157</v>
+        <v>0.1540090590015128</v>
       </c>
     </row>
     <row r="41">
@@ -1412,25 +1412,25 @@
         <v>1989</v>
       </c>
       <c r="B41" s="15" t="n">
-        <v>0.2368645091091621</v>
+        <v>0.2272089985012069</v>
       </c>
       <c r="C41" s="15" t="n">
-        <v>0.4076481022018533</v>
+        <v>0.3940104536936824</v>
       </c>
       <c r="D41" s="15" t="n">
-        <v>0.4488317975325229</v>
+        <v>0.4316231498727383</v>
       </c>
       <c r="E41" s="15" t="n">
-        <v>0.4355022682978007</v>
+        <v>0.4260029090095925</v>
       </c>
       <c r="F41" s="15" t="n">
-        <v>0.6793451181250911</v>
+        <v>0.6423018638851533</v>
       </c>
       <c r="G41" s="15" t="n">
-        <v>0.6793451181250909</v>
+        <v>0.6423018638851533</v>
       </c>
       <c r="H41" s="15" t="n">
-        <v>0.2012677781098609</v>
+        <v>0.1924488598707212</v>
       </c>
     </row>
     <row r="42">
@@ -1438,25 +1438,25 @@
         <v>1990</v>
       </c>
       <c r="B42" s="16" t="n">
-        <v>-0.03001740915118978</v>
+        <v>-0.02686455497420492</v>
       </c>
       <c r="C42" s="16" t="n">
-        <v>-0.05198888894256381</v>
+        <v>-0.04780037580080377</v>
       </c>
       <c r="D42" s="16" t="n">
-        <v>-0.1295947859430874</v>
+        <v>-0.1217451426862551</v>
       </c>
       <c r="E42" s="16" t="n">
-        <v>-0.2241107035601365</v>
+        <v>-0.2172093425855407</v>
       </c>
       <c r="F42" s="16" t="n">
-        <v>-0.479103160634812</v>
+        <v>-0.4636589594432232</v>
       </c>
       <c r="G42" s="16" t="n">
-        <v>-0.5052791049588621</v>
+        <v>-0.4906110009135206</v>
       </c>
       <c r="H42" s="16" t="n">
-        <v>-0.1861528461437714</v>
+        <v>-0.1781002685514583</v>
       </c>
     </row>
     <row r="43">
@@ -1464,10 +1464,10 @@
         <v>1991</v>
       </c>
       <c r="B43" s="15" t="n">
-        <v>0.3020291918806405</v>
+        <v>0.3052175307131875</v>
       </c>
       <c r="C43" s="15" t="n">
-        <v>0.5477588244412317</v>
+        <v>0.5500517979734378</v>
       </c>
       <c r="D43" s="15" t="n">
         <v>0.8652924905122881</v>
@@ -1479,10 +1479,10 @@
         <v>1.235286181188468</v>
       </c>
       <c r="G43" s="15" t="n">
-        <v>2.620657776071494</v>
+        <v>2.574041712079904</v>
       </c>
       <c r="H43" s="15" t="n">
-        <v>0.5753358626973928</v>
+        <v>0.5685929529778371</v>
       </c>
     </row>
     <row r="44">
@@ -1490,25 +1490,25 @@
         <v>1992</v>
       </c>
       <c r="B44" s="15" t="n">
-        <v>0.1684665400272747</v>
+        <v>0.1665996899649919</v>
       </c>
       <c r="C44" s="15" t="n">
-        <v>0.2976105281223074</v>
+        <v>0.2971087862665462</v>
       </c>
       <c r="D44" s="15" t="n">
-        <v>0.4550615141163856</v>
+        <v>0.4557061958415698</v>
       </c>
       <c r="E44" s="15" t="n">
-        <v>0.2241270760162706</v>
+        <v>0.224519648814487</v>
       </c>
       <c r="F44" s="15" t="n">
-        <v>0.4492558294916964</v>
+        <v>0.45002192007574</v>
       </c>
       <c r="G44" s="15" t="n">
-        <v>0.4492558294916982</v>
+        <v>0.4500219200757416</v>
       </c>
       <c r="H44" s="15" t="n">
-        <v>0.1543183530534227</v>
+        <v>0.1545348787862986</v>
       </c>
     </row>
     <row r="45">
@@ -1516,25 +1516,25 @@
         <v>1993</v>
       </c>
       <c r="B45" s="15" t="n">
-        <v>0.1142411357771667</v>
+        <v>0.1076362536613749</v>
       </c>
       <c r="C45" s="15" t="n">
-        <v>0.09279345267959925</v>
+        <v>0.07458021464130438</v>
       </c>
       <c r="D45" s="15" t="n">
-        <v>0.03991595564899098</v>
+        <v>0.01614640026870684</v>
       </c>
       <c r="E45" s="15" t="n">
-        <v>0.1001567035105535</v>
+        <v>0.07501021398028684</v>
       </c>
       <c r="F45" s="15" t="n">
-        <v>0.472122089343886</v>
+        <v>0.43847351674615</v>
       </c>
       <c r="G45" s="15" t="n">
-        <v>0.472122089343886</v>
+        <v>0.43847351674615</v>
       </c>
       <c r="H45" s="15" t="n">
-        <v>0.1562965196123225</v>
+        <v>0.147499777280453</v>
       </c>
     </row>
     <row r="46">
@@ -1542,25 +1542,25 @@
         <v>1994</v>
       </c>
       <c r="B46" s="16" t="n">
-        <v>-0.02337931746423627</v>
-      </c>
-      <c r="C46" s="15" t="n">
-        <v>0.000807746148752563</v>
-      </c>
-      <c r="D46" s="15" t="n">
-        <v>0.001820323248828748</v>
-      </c>
-      <c r="E46" s="15" t="n">
-        <v>0.006614724532152838</v>
+        <v>-0.02950273260943581</v>
+      </c>
+      <c r="C46" s="16" t="n">
+        <v>-0.007032439301531079</v>
+      </c>
+      <c r="D46" s="16" t="n">
+        <v>-0.008687537033379766</v>
+      </c>
+      <c r="E46" s="16" t="n">
+        <v>-0.009934599576893575</v>
       </c>
       <c r="F46" s="16" t="n">
-        <v>-0.1157615659215692</v>
+        <v>-0.1364178266499546</v>
       </c>
       <c r="G46" s="16" t="n">
-        <v>-0.1157615659215691</v>
+        <v>-0.1364178266499545</v>
       </c>
       <c r="H46" s="16" t="n">
-        <v>-0.02439149379324945</v>
+        <v>-0.031977299670092</v>
       </c>
     </row>
     <row r="47">
@@ -1568,25 +1568,25 @@
         <v>1995</v>
       </c>
       <c r="B47" s="15" t="n">
-        <v>0.474033862405748</v>
+        <v>0.4653528469230639</v>
       </c>
       <c r="C47" s="15" t="n">
-        <v>0.7383239100314505</v>
+        <v>0.7234453956502551</v>
       </c>
       <c r="D47" s="15" t="n">
-        <v>1.147746674392234</v>
+        <v>1.119553473211065</v>
       </c>
       <c r="E47" s="15" t="n">
-        <v>0.9095016003993112</v>
+        <v>0.886239703808146</v>
       </c>
       <c r="F47" s="15" t="n">
-        <v>1.660481983856468</v>
+        <v>1.57144423098257</v>
       </c>
       <c r="G47" s="15" t="n">
-        <v>1.660481983856469</v>
+        <v>1.57144423098257</v>
       </c>
       <c r="H47" s="15" t="n">
-        <v>0.4149519634011356</v>
+        <v>0.3991834329192567</v>
       </c>
     </row>
     <row r="48">
@@ -1594,25 +1594,25 @@
         <v>1996</v>
       </c>
       <c r="B48" s="15" t="n">
-        <v>0.1220414759097832</v>
+        <v>0.1239934425670413</v>
       </c>
       <c r="C48" s="15" t="n">
-        <v>0.2697423673546556</v>
+        <v>0.2724172919543411</v>
       </c>
       <c r="D48" s="15" t="n">
-        <v>0.4299464825265322</v>
+        <v>0.4338587518724679</v>
       </c>
       <c r="E48" s="15" t="n">
-        <v>0.3409024901147724</v>
+        <v>0.3493274435352733</v>
       </c>
       <c r="F48" s="15" t="n">
-        <v>0.672158597086342</v>
+        <v>0.7031884857409889</v>
       </c>
       <c r="G48" s="15" t="n">
-        <v>0.6721585970863408</v>
+        <v>0.7031884857409878</v>
       </c>
       <c r="H48" s="15" t="n">
-        <v>0.219505974336992</v>
+        <v>0.2270632173445144</v>
       </c>
     </row>
     <row r="49">
@@ -1620,25 +1620,25 @@
         <v>1997</v>
       </c>
       <c r="B49" s="15" t="n">
-        <v>0.282806760268389</v>
+        <v>0.2721841874108979</v>
       </c>
       <c r="C49" s="15" t="n">
-        <v>0.633947389718672</v>
+        <v>0.6173620694613529</v>
       </c>
       <c r="D49" s="15" t="n">
-        <v>0.9911374358416434</v>
+        <v>0.9632474168757765</v>
       </c>
       <c r="E49" s="15" t="n">
-        <v>0.9717476989320387</v>
+        <v>0.9536054642056768</v>
       </c>
       <c r="F49" s="15" t="n">
-        <v>0.6436993344866163</v>
+        <v>0.6041874365904263</v>
       </c>
       <c r="G49" s="15" t="n">
-        <v>0.6436993344866151</v>
+        <v>0.6041874365904252</v>
       </c>
       <c r="H49" s="15" t="n">
-        <v>0.2261654064824743</v>
+        <v>0.2163543377967392</v>
       </c>
     </row>
     <row r="50">
@@ -1646,25 +1646,25 @@
         <v>1998</v>
       </c>
       <c r="B50" s="15" t="n">
-        <v>0.319087570794957</v>
+        <v>0.3253709819734303</v>
       </c>
       <c r="C50" s="15" t="n">
-        <v>0.6835741044948311</v>
+        <v>0.6924616869454528</v>
       </c>
       <c r="D50" s="15" t="n">
-        <v>0.8406039988536791</v>
+        <v>0.8529744447456642</v>
       </c>
       <c r="E50" s="15" t="n">
-        <v>0.6902698870083451</v>
+        <v>0.7148590897330089</v>
       </c>
       <c r="F50" s="15" t="n">
-        <v>0.2145547811348878</v>
+        <v>0.240454275842977</v>
       </c>
       <c r="G50" s="15" t="n">
-        <v>1.128941083466231</v>
+        <v>1.174339199040356</v>
       </c>
       <c r="H50" s="15" t="n">
-        <v>0.3864358569191606</v>
+        <v>0.3963065396321566</v>
       </c>
     </row>
     <row r="51">
@@ -1672,25 +1672,25 @@
         <v>1999</v>
       </c>
       <c r="B51" s="15" t="n">
-        <v>0.5534856047379551</v>
+        <v>0.5661043833464285</v>
       </c>
       <c r="C51" s="15" t="n">
-        <v>1.322614638780552</v>
+        <v>1.35875267377596</v>
       </c>
       <c r="D51" s="15" t="n">
-        <v>2.147581131823013</v>
+        <v>2.213621488235486</v>
       </c>
       <c r="E51" s="15" t="n">
-        <v>1.421624751140155</v>
+        <v>1.472433596080058</v>
       </c>
       <c r="F51" s="15" t="n">
-        <v>3.947844227873866</v>
+        <v>4.051656451482201</v>
       </c>
       <c r="G51" s="15" t="n">
-        <v>3.947844227873868</v>
+        <v>4.051656451482202</v>
       </c>
       <c r="H51" s="15" t="n">
-        <v>0.8429428539642675</v>
+        <v>0.8558529333810629</v>
       </c>
     </row>
     <row r="52">
@@ -1698,25 +1698,25 @@
         <v>2000</v>
       </c>
       <c r="B52" s="15" t="n">
-        <v>0.07292176905944658</v>
-      </c>
-      <c r="C52" s="16" t="n">
-        <v>-0.03233166332120618</v>
+        <v>0.09365568667696843</v>
+      </c>
+      <c r="C52" s="15" t="n">
+        <v>0.002627304396334518</v>
       </c>
       <c r="D52" s="16" t="n">
-        <v>-0.08614453120215426</v>
+        <v>-0.04451311860812989</v>
       </c>
       <c r="E52" s="16" t="n">
-        <v>-0.1595426143848517</v>
+        <v>-0.1286226844361764</v>
       </c>
       <c r="F52" s="16" t="n">
-        <v>-0.3670832155791248</v>
+        <v>-0.3382501881589679</v>
       </c>
       <c r="G52" s="16" t="n">
-        <v>-0.8969672477188233</v>
+        <v>-0.8922735087553108</v>
       </c>
       <c r="H52" s="16" t="n">
-        <v>-0.4019776385253038</v>
+        <v>-0.3928897075473502</v>
       </c>
     </row>
     <row r="53">
@@ -1724,10 +1724,10 @@
         <v>2001</v>
       </c>
       <c r="B53" s="15" t="n">
-        <v>0.02546111480943014</v>
+        <v>0.02640696388800201</v>
       </c>
       <c r="C53" s="15" t="n">
-        <v>0.01612713543262934</v>
+        <v>0.01548503646299437</v>
       </c>
       <c r="D53" s="15" t="n">
         <v>0</v>
@@ -1739,10 +1739,10 @@
         <v>0</v>
       </c>
       <c r="G53" s="16" t="n">
-        <v>-0.640689271894741</v>
+        <v>-0.7186540577293372</v>
       </c>
       <c r="H53" s="16" t="n">
-        <v>-0.1489881873492552</v>
+        <v>-0.2105305732353466</v>
       </c>
     </row>
     <row r="54">
@@ -1750,10 +1750,10 @@
         <v>2002</v>
       </c>
       <c r="B54" s="15" t="n">
-        <v>0.1231764040292072</v>
+        <v>0.1200526873428713</v>
       </c>
       <c r="C54" s="15" t="n">
-        <v>0.1045813276735002</v>
+        <v>0.1026686845682971</v>
       </c>
       <c r="D54" s="15" t="n">
         <v>0</v>
@@ -1765,10 +1765,10 @@
         <v>0</v>
       </c>
       <c r="G54" s="16" t="n">
-        <v>-0.7857726628563829</v>
+        <v>-0.7762735338912158</v>
       </c>
       <c r="H54" s="16" t="n">
-        <v>-0.3252444057092333</v>
+        <v>-0.3152635389836316</v>
       </c>
     </row>
     <row r="55">
@@ -1776,10 +1776,10 @@
         <v>2003</v>
       </c>
       <c r="B55" s="15" t="n">
-        <v>0.3952357888846181</v>
+        <v>0.3861733150798568</v>
       </c>
       <c r="C55" s="15" t="n">
-        <v>0.6758601864258051</v>
+        <v>0.6681870519649238</v>
       </c>
       <c r="D55" s="15" t="n">
         <v>0.99277512546135</v>
@@ -1791,10 +1791,10 @@
         <v>1.755318413937077</v>
       </c>
       <c r="G55" s="15" t="n">
-        <v>1.597159647534639</v>
+        <v>1.884924570807031</v>
       </c>
       <c r="H55" s="15" t="n">
-        <v>0.4466332308330847</v>
+        <v>0.500078606674015</v>
       </c>
     </row>
     <row r="56">
@@ -1802,25 +1802,25 @@
         <v>2004</v>
       </c>
       <c r="B56" s="15" t="n">
-        <v>0.06457624224522407</v>
+        <v>0.06298366810082157</v>
       </c>
       <c r="C56" s="15" t="n">
-        <v>0.1072090738323244</v>
+        <v>0.1082283529339987</v>
       </c>
       <c r="D56" s="15" t="n">
-        <v>0.06421606563708138</v>
+        <v>0.06764548510048485</v>
       </c>
       <c r="E56" s="15" t="n">
-        <v>0.05488762327001728</v>
+        <v>0.05896206814990923</v>
       </c>
       <c r="F56" s="16" t="n">
-        <v>-0.2048427239977068</v>
+        <v>-0.2009284752945831</v>
       </c>
       <c r="G56" s="15" t="n">
-        <v>0.1588657522350321</v>
+        <v>0.1645703957120885</v>
       </c>
       <c r="H56" s="15" t="n">
-        <v>0.08409905040098643</v>
+        <v>0.08589024814659861</v>
       </c>
     </row>
     <row r="57">
@@ -1828,25 +1828,25 @@
         <v>2005</v>
       </c>
       <c r="B57" s="15" t="n">
-        <v>0.08479849396683159</v>
+        <v>0.06620847250066597</v>
       </c>
       <c r="C57" s="15" t="n">
-        <v>0.05787733284865593</v>
-      </c>
-      <c r="D57" s="15" t="n">
-        <v>0.01916828264139769</v>
+        <v>0.03032357837003397</v>
+      </c>
+      <c r="D57" s="16" t="n">
+        <v>-0.0121529109892613</v>
       </c>
       <c r="E57" s="15" t="n">
-        <v>0.08298004084154975</v>
-      </c>
-      <c r="F57" s="15" t="n">
-        <v>0.01834219832836625</v>
-      </c>
-      <c r="G57" s="15" t="n">
-        <v>0.01834219832836648</v>
+        <v>0.04816025911503252</v>
+      </c>
+      <c r="F57" s="16" t="n">
+        <v>-0.01439935897784395</v>
+      </c>
+      <c r="G57" s="16" t="n">
+        <v>-0.01439935897784372</v>
       </c>
       <c r="H57" s="15" t="n">
-        <v>0.02470560528826948</v>
+        <v>0.01373521118044052</v>
       </c>
     </row>
     <row r="58">
@@ -1854,25 +1854,25 @@
         <v>2006</v>
       </c>
       <c r="B58" s="15" t="n">
-        <v>0.2261427575512125</v>
+        <v>0.2583595130601297</v>
       </c>
       <c r="C58" s="15" t="n">
-        <v>0.3500264505313411</v>
+        <v>0.4075075854559312</v>
       </c>
       <c r="D58" s="15" t="n">
-        <v>0.451703909161656</v>
+        <v>0.5275268242666009</v>
       </c>
       <c r="E58" s="15" t="n">
-        <v>0.140497565305969</v>
+        <v>0.1902055975229084</v>
       </c>
       <c r="F58" s="15" t="n">
-        <v>0.1659660296818448</v>
+        <v>0.2268647726871389</v>
       </c>
       <c r="G58" s="15" t="n">
-        <v>0.1659660296818486</v>
+        <v>0.2268647726871429</v>
       </c>
       <c r="H58" s="15" t="n">
-        <v>0.07645718744799845</v>
+        <v>0.09521065628828262</v>
       </c>
     </row>
     <row r="59">
@@ -1880,25 +1880,25 @@
         <v>2007</v>
       </c>
       <c r="B59" s="15" t="n">
-        <v>0.1793393772076162</v>
+        <v>0.1799830895089312</v>
       </c>
       <c r="C59" s="15" t="n">
-        <v>0.1730232908912228</v>
+        <v>0.1796582690292347</v>
       </c>
       <c r="D59" s="15" t="n">
-        <v>0.1233882235717694</v>
+        <v>0.1340851575566344</v>
       </c>
       <c r="E59" s="15" t="n">
-        <v>0.09004432308559875</v>
+        <v>0.09869130915437217</v>
       </c>
       <c r="F59" s="15" t="n">
-        <v>0.1870216548593122</v>
+        <v>0.1985843601442481</v>
       </c>
       <c r="G59" s="15" t="n">
-        <v>0.1870216548593129</v>
+        <v>0.1985843601442485</v>
       </c>
       <c r="H59" s="15" t="n">
-        <v>0.09455427017645392</v>
+        <v>0.09812071683867864</v>
       </c>
     </row>
     <row r="60">
@@ -1906,25 +1906,25 @@
         <v>2008</v>
       </c>
       <c r="B60" s="15" t="n">
-        <v>0.05357928874278906</v>
+        <v>0.05881552169961091</v>
       </c>
       <c r="C60" s="15" t="n">
-        <v>0.03072917149641441</v>
+        <v>0.02704759742690022</v>
       </c>
       <c r="D60" s="16" t="n">
-        <v>-0.06151023211291462</v>
+        <v>-0.07947835675457104</v>
       </c>
       <c r="E60" s="16" t="n">
-        <v>-0.1186511371738179</v>
+        <v>-0.1537563440587768</v>
       </c>
       <c r="F60" s="16" t="n">
-        <v>-0.331940413973785</v>
+        <v>-0.3641915279832347</v>
       </c>
       <c r="G60" s="16" t="n">
-        <v>-0.8699301787523726</v>
+        <v>-0.8762094040220798</v>
       </c>
       <c r="H60" s="16" t="n">
-        <v>-0.3956882394421908</v>
+        <v>-0.4054059104782409</v>
       </c>
     </row>
     <row r="61">
@@ -1932,10 +1932,10 @@
         <v>2009</v>
       </c>
       <c r="B61" s="15" t="n">
-        <v>0.2228436267392762</v>
+        <v>0.2156669096838011</v>
       </c>
       <c r="C61" s="15" t="n">
-        <v>0.4327369985388894</v>
+        <v>0.4267548075148984</v>
       </c>
       <c r="D61" s="15" t="n">
         <v>0.5432225225653364</v>
@@ -1947,10 +1947,10 @@
         <v>0.5917514957012741</v>
       </c>
       <c r="G61" s="15" t="n">
-        <v>1.103900622020674</v>
+        <v>1.324673874880211</v>
       </c>
       <c r="H61" s="15" t="n">
-        <v>0.390231622290657</v>
+        <v>0.4388755193449778</v>
       </c>
     </row>
     <row r="62">
@@ -1958,25 +1958,25 @@
         <v>2010</v>
       </c>
       <c r="B62" s="15" t="n">
-        <v>0.1937389275809147</v>
+        <v>0.2227644766911345</v>
       </c>
       <c r="C62" s="15" t="n">
-        <v>0.3023153104457659</v>
+        <v>0.3544635142269217</v>
       </c>
       <c r="D62" s="15" t="n">
-        <v>0.203447685358058</v>
+        <v>0.2618094703587007</v>
       </c>
       <c r="E62" s="15" t="n">
-        <v>0.3610884027847234</v>
+        <v>0.4316397769775931</v>
       </c>
       <c r="F62" s="15" t="n">
-        <v>0.3394088678086455</v>
+        <v>0.4089027853914853</v>
       </c>
       <c r="G62" s="15" t="n">
-        <v>0.3394088678086433</v>
+        <v>0.4089027853914826</v>
       </c>
       <c r="H62" s="15" t="n">
-        <v>0.1492147038401792</v>
+        <v>0.1691030701240997</v>
       </c>
     </row>
     <row r="63">
@@ -1984,25 +1984,25 @@
         <v>2011</v>
       </c>
       <c r="B63" s="16" t="n">
-        <v>-0.03101250483907803</v>
+        <v>-0.01940321484245444</v>
       </c>
       <c r="C63" s="16" t="n">
-        <v>-0.1491924803278044</v>
+        <v>-0.1265113932269826</v>
       </c>
       <c r="D63" s="16" t="n">
-        <v>-0.2765712428625557</v>
+        <v>-0.2507263406918773</v>
       </c>
       <c r="E63" s="16" t="n">
-        <v>-0.3069628750778119</v>
+        <v>-0.2841290593495269</v>
       </c>
       <c r="F63" s="16" t="n">
-        <v>-0.4396468792296196</v>
+        <v>-0.4151744975591524</v>
       </c>
       <c r="G63" s="16" t="n">
-        <v>-0.2592159470618752</v>
+        <v>-0.2268635795869269</v>
       </c>
       <c r="H63" s="16" t="n">
-        <v>-0.032089717839067</v>
+        <v>-0.01798814600616949</v>
       </c>
     </row>
     <row r="64">
@@ -2010,25 +2010,25 @@
         <v>2012</v>
       </c>
       <c r="B64" s="15" t="n">
-        <v>0.1646020169450002</v>
+        <v>0.1891451512998973</v>
       </c>
       <c r="C64" s="15" t="n">
-        <v>0.2701227754305102</v>
+        <v>0.3200129485359837</v>
       </c>
       <c r="D64" s="15" t="n">
-        <v>0.3457831232986064</v>
+        <v>0.4132602164271597</v>
       </c>
       <c r="E64" s="15" t="n">
-        <v>0.224538839937545</v>
+        <v>0.2738004568343584</v>
       </c>
       <c r="F64" s="15" t="n">
-        <v>0.3751955232610551</v>
+        <v>0.4441473437933345</v>
       </c>
       <c r="G64" s="15" t="n">
-        <v>0.3751955232610551</v>
+        <v>0.4441473437933345</v>
       </c>
       <c r="H64" s="15" t="n">
-        <v>0.1399883879986044</v>
+        <v>0.1590542285808168</v>
       </c>
     </row>
     <row r="65">
@@ -2036,25 +2036,25 @@
         <v>2013</v>
       </c>
       <c r="B65" s="15" t="n">
-        <v>0.07932102608585367</v>
+        <v>0.09819012134405725</v>
       </c>
       <c r="C65" s="15" t="n">
-        <v>0.3000844473287276</v>
+        <v>0.3318676102978755</v>
       </c>
       <c r="D65" s="15" t="n">
-        <v>0.6847529155635729</v>
+        <v>0.7666927557492802</v>
       </c>
       <c r="E65" s="15" t="n">
-        <v>0.7973708527127319</v>
+        <v>0.847041152680321</v>
       </c>
       <c r="F65" s="15" t="n">
-        <v>1.294292129575793</v>
+        <v>1.505634487623038</v>
       </c>
       <c r="G65" s="15" t="n">
-        <v>1.294292129575797</v>
+        <v>1.505634487623041</v>
       </c>
       <c r="H65" s="15" t="n">
-        <v>0.3419797287438076</v>
+        <v>0.3832011916396991</v>
       </c>
     </row>
     <row r="66">
@@ -2062,25 +2062,25 @@
         <v>2014</v>
       </c>
       <c r="B66" s="15" t="n">
-        <v>0.05719213571127568</v>
+        <v>0.05446936988546858</v>
       </c>
       <c r="C66" s="15" t="n">
-        <v>0.05431874772477996</v>
+        <v>0.0398356493645784</v>
       </c>
       <c r="D66" s="15" t="n">
-        <v>0.1056480884247872</v>
+        <v>0.07898958587284111</v>
       </c>
       <c r="E66" s="15" t="n">
-        <v>0.1038358087694473</v>
+        <v>0.07722100245532104</v>
       </c>
       <c r="F66" s="15" t="n">
-        <v>0.3943631388173678</v>
+        <v>0.3607433698477851</v>
       </c>
       <c r="G66" s="15" t="n">
-        <v>0.3943631388173681</v>
+        <v>0.3607433698477853</v>
       </c>
       <c r="H66" s="15" t="n">
-        <v>0.1431257512400543</v>
+        <v>0.1339513770555441</v>
       </c>
     </row>
     <row r="67">
@@ -2088,25 +2088,25 @@
         <v>2015</v>
       </c>
       <c r="B67" s="16" t="n">
-        <v>-0.07270277871044639</v>
+        <v>-0.07276994449154717</v>
       </c>
       <c r="C67" s="16" t="n">
-        <v>-0.1126271873401637</v>
+        <v>-0.1151410709672913</v>
       </c>
       <c r="D67" s="16" t="n">
-        <v>-0.132489387497705</v>
+        <v>-0.1369020782663063</v>
       </c>
       <c r="E67" s="15" t="n">
-        <v>0.03664578305453658</v>
+        <v>0.03090607817109969</v>
       </c>
       <c r="F67" s="15" t="n">
-        <v>0.08207295091035594</v>
+        <v>0.07570284687617312</v>
       </c>
       <c r="G67" s="15" t="n">
-        <v>0.08207295091035614</v>
+        <v>0.07570284687617312</v>
       </c>
       <c r="H67" s="15" t="n">
-        <v>0.05936352286162361</v>
+        <v>0.05729676886284363</v>
       </c>
     </row>
     <row r="68">
@@ -2114,25 +2114,25 @@
         <v>2016</v>
       </c>
       <c r="B68" s="15" t="n">
-        <v>0.03308994685015842</v>
+        <v>0.01867511255396792</v>
       </c>
       <c r="C68" s="15" t="n">
-        <v>0.05527610730809851</v>
-      </c>
-      <c r="D68" s="15" t="n">
-        <v>0.001328323048628732</v>
+        <v>0.02233331962874807</v>
+      </c>
+      <c r="D68" s="16" t="n">
+        <v>-0.05227806871659989</v>
       </c>
       <c r="E68" s="16" t="n">
-        <v>-0.000879072663356517</v>
+        <v>-0.03476283893789955</v>
       </c>
       <c r="F68" s="16" t="n">
-        <v>-0.1371979524737815</v>
+        <v>-0.1911521464202265</v>
       </c>
       <c r="G68" s="15" t="n">
-        <v>0.2167977351420303</v>
+        <v>0.1407068853536226</v>
       </c>
       <c r="H68" s="15" t="n">
-        <v>0.09790362572846224</v>
+        <v>0.07503079422200232</v>
       </c>
     </row>
     <row r="69">
@@ -2140,25 +2140,25 @@
         <v>2017</v>
       </c>
       <c r="B69" s="15" t="n">
-        <v>0.2035197759914718</v>
+        <v>0.2152068114952526</v>
       </c>
       <c r="C69" s="15" t="n">
-        <v>0.3124982085089512</v>
+        <v>0.3329804758130857</v>
       </c>
       <c r="D69" s="15" t="n">
-        <v>0.4652034605940945</v>
+        <v>0.4953903838713161</v>
       </c>
       <c r="E69" s="15" t="n">
-        <v>0.363178493904309</v>
+        <v>0.3898825530142414</v>
       </c>
       <c r="F69" s="15" t="n">
-        <v>0.9821004829237668</v>
+        <v>1.032801125999219</v>
       </c>
       <c r="G69" s="15" t="n">
-        <v>0.9821004829237664</v>
+        <v>1.032801125999218</v>
       </c>
       <c r="H69" s="15" t="n">
-        <v>0.2715579873235385</v>
+        <v>0.2824142852021743</v>
       </c>
     </row>
     <row r="70">
@@ -2166,25 +2166,25 @@
         <v>2018</v>
       </c>
       <c r="B70" s="15" t="n">
-        <v>0.008768898318487484</v>
+        <v>0.02226735897456278</v>
       </c>
       <c r="C70" s="15" t="n">
-        <v>0.0748875043935362</v>
+        <v>0.100598416988714</v>
       </c>
       <c r="D70" s="15" t="n">
-        <v>0.02083430136115272</v>
+        <v>0.05952629287363354</v>
       </c>
       <c r="E70" s="16" t="n">
-        <v>-0.1209748452753411</v>
+        <v>-0.1030168510136859</v>
       </c>
       <c r="F70" s="16" t="n">
-        <v>-0.2872912212926608</v>
+        <v>-0.2552563743843378</v>
       </c>
       <c r="G70" s="16" t="n">
-        <v>-0.2619173864108884</v>
+        <v>-0.2287420359193361</v>
       </c>
       <c r="H70" s="16" t="n">
-        <v>-0.05303631023670352</v>
+        <v>-0.03883749095433742</v>
       </c>
     </row>
     <row r="71">
@@ -2192,10 +2192,10 @@
         <v>2019</v>
       </c>
       <c r="B71" s="15" t="n">
-        <v>0.2467381492315928</v>
+        <v>0.248358638408362</v>
       </c>
       <c r="C71" s="15" t="n">
-        <v>0.3802341097437396</v>
+        <v>0.3821679957955462</v>
       </c>
       <c r="D71" s="15" t="n">
         <v>0.4761379368410685</v>
@@ -2207,10 +2207,10 @@
         <v>0.612044898421809</v>
       </c>
       <c r="G71" s="15" t="n">
-        <v>1.243840792951809</v>
+        <v>1.274869089109652</v>
       </c>
       <c r="H71" s="15" t="n">
-        <v>0.3460366712595921</v>
+        <v>0.3522564081297441</v>
       </c>
     </row>
     <row r="72">
@@ -2218,25 +2218,25 @@
         <v>2020</v>
       </c>
       <c r="B72" s="15" t="n">
-        <v>0.3097633149128773</v>
+        <v>0.3309956495938287</v>
       </c>
       <c r="C72" s="15" t="n">
-        <v>0.5718796761327414</v>
+        <v>0.6204657761335497</v>
       </c>
       <c r="D72" s="15" t="n">
-        <v>0.6202654284863043</v>
+        <v>0.6848733699986262</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>0.6443038148434969</v>
+        <v>0.6808034670476311</v>
       </c>
       <c r="F72" s="15" t="n">
-        <v>0.786337385972333</v>
+        <v>0.857703734772127</v>
       </c>
       <c r="G72" s="15" t="n">
-        <v>0.8847833413119304</v>
+        <v>0.9600827256300238</v>
       </c>
       <c r="H72" s="15" t="n">
-        <v>0.4175110356768008</v>
+        <v>0.4364042568078441</v>
       </c>
     </row>
     <row r="73">
@@ -2244,25 +2244,25 @@
         <v>2021</v>
       </c>
       <c r="B73" s="15" t="n">
-        <v>0.1159067181207105</v>
+        <v>0.1104391361025869</v>
       </c>
       <c r="C73" s="15" t="n">
-        <v>0.2881129415652957</v>
+        <v>0.2574752818710651</v>
       </c>
       <c r="D73" s="15" t="n">
-        <v>0.4565059427943541</v>
+        <v>0.4037643767197108</v>
       </c>
       <c r="E73" s="15" t="n">
-        <v>0.2814546064980841</v>
+        <v>0.2247876578555364</v>
       </c>
       <c r="F73" s="15" t="n">
-        <v>0.6823012453837123</v>
+        <v>0.6079085374484934</v>
       </c>
       <c r="G73" s="15" t="n">
-        <v>0.682301245383712</v>
+        <v>0.6079085374484929</v>
       </c>
       <c r="H73" s="15" t="n">
-        <v>0.2320377279364918</v>
+        <v>0.21389117827749</v>
       </c>
     </row>
     <row r="74">
@@ -2270,25 +2270,25 @@
         <v>2022</v>
       </c>
       <c r="B74" s="16" t="n">
-        <v>-0.08744768992489049</v>
+        <v>-0.08449030896673904</v>
       </c>
       <c r="C74" s="16" t="n">
-        <v>-0.1244295010032444</v>
+        <v>-0.108779177738955</v>
       </c>
       <c r="D74" s="16" t="n">
-        <v>-0.1440932414313002</v>
+        <v>-0.1176258515769151</v>
       </c>
       <c r="E74" s="16" t="n">
-        <v>-0.214865299334692</v>
+        <v>-0.1940883389413854</v>
       </c>
       <c r="F74" s="16" t="n">
-        <v>-0.4103953986477075</v>
+        <v>-0.389179529157927</v>
       </c>
       <c r="G74" s="16" t="n">
-        <v>-0.7896456717483915</v>
+        <v>-0.7820764466023177</v>
       </c>
       <c r="H74" s="16" t="n">
-        <v>-0.3389368527446884</v>
+        <v>-0.3310002734629972</v>
       </c>
     </row>
     <row r="75">
@@ -2296,10 +2296,10 @@
         <v>2023</v>
       </c>
       <c r="B75" s="15" t="n">
-        <v>0.2386260724851592</v>
+        <v>0.2454271463908682</v>
       </c>
       <c r="C75" s="15" t="n">
-        <v>0.3968244600624387</v>
+        <v>0.4030314751076863</v>
       </c>
       <c r="D75" s="15" t="n">
         <v>0.5138054298081998</v>
@@ -2311,10 +2311,10 @@
         <v>0.8492043697015528</v>
       </c>
       <c r="G75" s="15" t="n">
-        <v>1.734984397750709</v>
+        <v>1.672568890619622</v>
       </c>
       <c r="H75" s="15" t="n">
-        <v>0.4452082252910512</v>
+        <v>0.4342308910998991</v>
       </c>
     </row>
     <row r="76">
@@ -2322,25 +2322,25 @@
         <v>2024</v>
       </c>
       <c r="B76" s="15" t="n">
-        <v>0.1964308118985447</v>
+        <v>0.1764909525877734</v>
       </c>
       <c r="C76" s="15" t="n">
-        <v>0.3000377168930617</v>
+        <v>0.2575531954636097</v>
       </c>
       <c r="D76" s="15" t="n">
-        <v>0.3170037438878803</v>
+        <v>0.2605117095441229</v>
       </c>
       <c r="E76" s="15" t="n">
-        <v>0.3595862367157499</v>
+        <v>0.3030947421724088</v>
       </c>
       <c r="F76" s="15" t="n">
-        <v>1.00949446850217</v>
+        <v>0.9108707834937771</v>
       </c>
       <c r="G76" s="15" t="n">
-        <v>1.009494468502171</v>
+        <v>0.9108707834937778</v>
       </c>
       <c r="H76" s="15" t="n">
-        <v>0.3077926972856336</v>
+        <v>0.2864125854773165</v>
       </c>
     </row>
     <row r="77">
@@ -2348,25 +2348,25 @@
         <v>2025</v>
       </c>
       <c r="B77" s="15" t="n">
-        <v>0.3234156621082722</v>
+        <v>0.3268440831233055</v>
       </c>
       <c r="C77" s="15" t="n">
-        <v>0.3697321290792874</v>
+        <v>0.3714167118536076</v>
       </c>
       <c r="D77" s="15" t="n">
-        <v>0.2936026495778305</v>
+        <v>0.2902467751719067</v>
       </c>
       <c r="E77" s="15" t="n">
-        <v>0.1353410766137213</v>
+        <v>0.1321573527509299</v>
       </c>
       <c r="F77" s="16" t="n">
-        <v>-0.1379701827899386</v>
+        <v>-0.1420171835270407</v>
       </c>
       <c r="G77" s="15" t="n">
-        <v>0.464161991907265</v>
+        <v>0.4572881407455232</v>
       </c>
       <c r="H77" s="15" t="n">
-        <v>0.2054480840506316</v>
+        <v>0.203575377430282</v>
       </c>
     </row>
     <row r="78">
@@ -2374,25 +2374,25 @@
         <v>2026</v>
       </c>
       <c r="B78" s="16" t="n">
-        <v>-0.03675308963186919</v>
+        <v>-0.03825769417685288</v>
       </c>
       <c r="C78" s="16" t="n">
-        <v>-0.08400093564001733</v>
+        <v>-0.08505296271368845</v>
       </c>
       <c r="D78" s="16" t="n">
-        <v>-0.1112000677432189</v>
+        <v>-0.1118534403426848</v>
       </c>
       <c r="E78" s="16" t="n">
-        <v>-0.1516931853693878</v>
+        <v>-0.1524184658834828</v>
       </c>
       <c r="F78" s="16" t="n">
-        <v>-0.2351409842729421</v>
+        <v>-0.2357949190646582</v>
       </c>
       <c r="G78" s="16" t="n">
-        <v>-0.235140984272942</v>
+        <v>-0.2357949190646581</v>
       </c>
       <c r="H78" s="16" t="n">
-        <v>-0.07865294436422099</v>
+        <v>-0.07890503944613314</v>
       </c>
     </row>
     <row r="80">
@@ -2450,26 +2450,26 @@
           <t>2021-01</t>
         </is>
       </c>
-      <c r="B82" s="15" t="n">
-        <v>0.004114578789393919</v>
+      <c r="B82" s="16" t="n">
+        <v>-0.000805257901230538</v>
       </c>
       <c r="C82" s="15" t="n">
-        <v>0.04205632415442473</v>
+        <v>0.01727110073848115</v>
       </c>
       <c r="D82" s="15" t="n">
-        <v>0.06735473167385786</v>
+        <v>0.02870472795491796</v>
       </c>
       <c r="E82" s="15" t="n">
-        <v>0.08024330909433285</v>
+        <v>0.03247408511441519</v>
       </c>
       <c r="F82" s="15" t="n">
-        <v>0.08024330909433219</v>
+        <v>0.03247408511441452</v>
       </c>
       <c r="G82" s="15" t="n">
-        <v>0.08024330909433264</v>
+        <v>0.03247408511441496</v>
       </c>
       <c r="H82" s="15" t="n">
-        <v>0.02931383194671833</v>
+        <v>0.01415318049702385</v>
       </c>
     </row>
     <row r="83">
@@ -2479,25 +2479,25 @@
         </is>
       </c>
       <c r="B83" s="16" t="n">
-        <v>-0.04559927012897647</v>
-      </c>
-      <c r="C83" s="16" t="n">
-        <v>-0.04604536121525782</v>
-      </c>
-      <c r="D83" s="16" t="n">
-        <v>-0.04350535555127511</v>
-      </c>
-      <c r="E83" s="16" t="n">
-        <v>-0.05664055715549098</v>
-      </c>
-      <c r="F83" s="16" t="n">
-        <v>-0.05508417748004801</v>
-      </c>
-      <c r="G83" s="16" t="n">
-        <v>-0.05508417748004824</v>
-      </c>
-      <c r="H83" s="16" t="n">
-        <v>-0.01574527373614709</v>
+        <v>-0.02105907489575109</v>
+      </c>
+      <c r="C83" s="15" t="n">
+        <v>0.0006755154592403829</v>
+      </c>
+      <c r="D83" s="15" t="n">
+        <v>0.01627755740598813</v>
+      </c>
+      <c r="E83" s="15" t="n">
+        <v>0.01536360007308235</v>
+      </c>
+      <c r="F83" s="15" t="n">
+        <v>0.01703877413565724</v>
+      </c>
+      <c r="G83" s="15" t="n">
+        <v>0.01703877413565702</v>
+      </c>
+      <c r="H83" s="15" t="n">
+        <v>0.009307785204732966</v>
       </c>
     </row>
     <row r="84">
@@ -2507,25 +2507,25 @@
         </is>
       </c>
       <c r="B84" s="16" t="n">
-        <v>-0.02371772270345485</v>
+        <v>-0.01069043328043029</v>
       </c>
       <c r="C84" s="16" t="n">
-        <v>-0.0303825220225078</v>
+        <v>-0.009659101653672232</v>
       </c>
       <c r="D84" s="16" t="n">
-        <v>-0.03860089904679764</v>
-      </c>
-      <c r="E84" s="16" t="n">
-        <v>-0.0169705022858232</v>
+        <v>-0.003911718342873516</v>
+      </c>
+      <c r="E84" s="15" t="n">
+        <v>0.003468387429306885</v>
       </c>
       <c r="F84" s="16" t="n">
-        <v>-0.0923701884814746</v>
+        <v>-0.01056794071054035</v>
       </c>
       <c r="G84" s="16" t="n">
-        <v>-0.09237018848147451</v>
-      </c>
-      <c r="H84" s="16" t="n">
-        <v>-0.02516478306352687</v>
+        <v>-0.01056794071054035</v>
+      </c>
+      <c r="H84" s="15" t="n">
+        <v>0.004132736746364385</v>
       </c>
     </row>
     <row r="85">
@@ -2535,25 +2535,25 @@
         </is>
       </c>
       <c r="B85" s="15" t="n">
-        <v>0.02249563346445749</v>
+        <v>0.03336905808268997</v>
       </c>
       <c r="C85" s="15" t="n">
-        <v>0.02835754348053343</v>
+        <v>0.04291060661675195</v>
       </c>
       <c r="D85" s="15" t="n">
-        <v>0.03895966029112707</v>
+        <v>0.05882264681228633</v>
       </c>
       <c r="E85" s="15" t="n">
-        <v>0.02223476877414021</v>
+        <v>0.03468323027351538</v>
       </c>
       <c r="F85" s="15" t="n">
-        <v>0.1053132757221209</v>
+        <v>0.1636599562893613</v>
       </c>
       <c r="G85" s="15" t="n">
-        <v>0.1053132757221207</v>
+        <v>0.1636599562893613</v>
       </c>
       <c r="H85" s="15" t="n">
-        <v>0.03579861910614146</v>
+        <v>0.05403612813274172</v>
       </c>
     </row>
     <row r="86">
@@ -2563,25 +2563,25 @@
         </is>
       </c>
       <c r="B86" s="15" t="n">
-        <v>0.001060852392591016</v>
+        <v>0.002691639112216037</v>
       </c>
       <c r="C86" s="16" t="n">
-        <v>-0.01792177941499218</v>
+        <v>-0.02078705993265451</v>
       </c>
       <c r="D86" s="16" t="n">
-        <v>-0.05150956129988571</v>
+        <v>-0.05934102256568385</v>
       </c>
       <c r="E86" s="16" t="n">
-        <v>-0.04737549843773548</v>
+        <v>-0.05405133641468762</v>
       </c>
       <c r="F86" s="16" t="n">
-        <v>-0.04085762790036485</v>
+        <v>-0.05481302766845476</v>
       </c>
       <c r="G86" s="16" t="n">
-        <v>-0.04085762790036485</v>
+        <v>-0.05481302766845476</v>
       </c>
       <c r="H86" s="16" t="n">
-        <v>-0.0105346252060039</v>
+        <v>-0.01532223458573412</v>
       </c>
     </row>
     <row r="87">
@@ -2591,25 +2591,25 @@
         </is>
       </c>
       <c r="B87" s="15" t="n">
-        <v>0.01639580095209459</v>
+        <v>0.01497839326644845</v>
       </c>
       <c r="C87" s="15" t="n">
-        <v>0.0525589396035937</v>
+        <v>0.0508402108297985</v>
       </c>
       <c r="D87" s="15" t="n">
-        <v>0.1006384135840477</v>
+        <v>0.09847653646198572</v>
       </c>
       <c r="E87" s="15" t="n">
-        <v>0.06518432516705919</v>
+        <v>0.06446751222092728</v>
       </c>
       <c r="F87" s="15" t="n">
-        <v>0.1729037964346636</v>
+        <v>0.1697261302473085</v>
       </c>
       <c r="G87" s="15" t="n">
-        <v>0.1729037964346631</v>
+        <v>0.1697261302473083</v>
       </c>
       <c r="H87" s="15" t="n">
-        <v>0.05587091455547633</v>
+        <v>0.05492939338902492</v>
       </c>
     </row>
     <row r="88">
@@ -2619,25 +2619,25 @@
         </is>
       </c>
       <c r="B88" s="15" t="n">
-        <v>0.02162293862734521</v>
+        <v>0.02291453123990728</v>
       </c>
       <c r="C88" s="15" t="n">
-        <v>0.02423883744675415</v>
+        <v>0.02707784317183925</v>
       </c>
       <c r="D88" s="15" t="n">
-        <v>0.02587205830313377</v>
+        <v>0.02953406508393664</v>
       </c>
       <c r="E88" s="15" t="n">
-        <v>0.02381554685928511</v>
+        <v>0.02712677481406089</v>
       </c>
       <c r="F88" s="15" t="n">
-        <v>0.02710861975564671</v>
+        <v>0.03098890600302773</v>
       </c>
       <c r="G88" s="15" t="n">
-        <v>0.02710861975564671</v>
+        <v>0.03098890600302773</v>
       </c>
       <c r="H88" s="15" t="n">
-        <v>0.01034952989112914</v>
+        <v>0.01163334746157862</v>
       </c>
     </row>
     <row r="89">
@@ -2647,25 +2647,25 @@
         </is>
       </c>
       <c r="B89" s="15" t="n">
-        <v>0.03752472233952808</v>
+        <v>0.04068185427512683</v>
       </c>
       <c r="C89" s="15" t="n">
-        <v>0.08255321791831548</v>
+        <v>0.08486140230876416</v>
       </c>
       <c r="D89" s="15" t="n">
-        <v>0.1121057734782489</v>
+        <v>0.1138726428444201</v>
       </c>
       <c r="E89" s="15" t="n">
-        <v>0.08041811459778515</v>
+        <v>0.08144807500588523</v>
       </c>
       <c r="F89" s="15" t="n">
-        <v>0.1187489523688758</v>
+        <v>0.1206300547572678</v>
       </c>
       <c r="G89" s="15" t="n">
-        <v>0.1187489523688758</v>
+        <v>0.1206300547572676</v>
       </c>
       <c r="H89" s="15" t="n">
-        <v>0.03938200073755693</v>
+        <v>0.03997637509763852</v>
       </c>
     </row>
     <row r="90">
@@ -2675,25 +2675,25 @@
         </is>
       </c>
       <c r="B90" s="16" t="n">
-        <v>-0.04575763414779965</v>
+        <v>-0.04252569622765767</v>
       </c>
       <c r="C90" s="16" t="n">
-        <v>-0.06607279891723328</v>
+        <v>-0.05953015197483048</v>
       </c>
       <c r="D90" s="16" t="n">
-        <v>-0.08720796942386932</v>
+        <v>-0.07873542449358739</v>
       </c>
       <c r="E90" s="16" t="n">
-        <v>-0.08455035307205128</v>
+        <v>-0.07685433561731592</v>
       </c>
       <c r="F90" s="16" t="n">
-        <v>-0.1648210905816921</v>
+        <v>-0.1566167627241118</v>
       </c>
       <c r="G90" s="16" t="n">
-        <v>-0.1648210905816923</v>
+        <v>-0.156616762724112</v>
       </c>
       <c r="H90" s="16" t="n">
-        <v>-0.05622695440812087</v>
+        <v>-0.05312585317477336</v>
       </c>
     </row>
     <row r="91">
@@ -2703,25 +2703,25 @@
         </is>
       </c>
       <c r="B91" s="15" t="n">
-        <v>0.03485641686033625</v>
+        <v>0.03911047872663431</v>
       </c>
       <c r="C91" s="15" t="n">
-        <v>0.06140912441528279</v>
+        <v>0.06670936028154539</v>
       </c>
       <c r="D91" s="15" t="n">
-        <v>0.09412202048240248</v>
+        <v>0.1023995407681799</v>
       </c>
       <c r="E91" s="15" t="n">
-        <v>0.07149401553131507</v>
+        <v>0.08128897902050468</v>
       </c>
       <c r="F91" s="15" t="n">
-        <v>0.1974756469913186</v>
+        <v>0.2268036107035201</v>
       </c>
       <c r="G91" s="15" t="n">
-        <v>0.1974756469913186</v>
+        <v>0.2268036107035201</v>
       </c>
       <c r="H91" s="15" t="n">
-        <v>0.06396022713674121</v>
+        <v>0.07265832106934167</v>
       </c>
     </row>
     <row r="92">
@@ -2731,25 +2731,25 @@
         </is>
       </c>
       <c r="B92" s="15" t="n">
-        <v>0.01239862798718305</v>
+        <v>0.01927176352759031</v>
       </c>
       <c r="C92" s="15" t="n">
-        <v>0.02342874962531361</v>
+        <v>0.03475327067679035</v>
       </c>
       <c r="D92" s="15" t="n">
-        <v>0.03474638898500681</v>
+        <v>0.04966229732321414</v>
       </c>
       <c r="E92" s="15" t="n">
-        <v>0.000826407602200429</v>
-      </c>
-      <c r="F92" s="16" t="n">
-        <v>-0.01793557470542684</v>
-      </c>
-      <c r="G92" s="16" t="n">
-        <v>-0.01793557470542684</v>
-      </c>
-      <c r="H92" s="16" t="n">
-        <v>-0.003733636263791418</v>
+        <v>0.007865958424170261</v>
+      </c>
+      <c r="F92" s="15" t="n">
+        <v>0.000571096979138374</v>
+      </c>
+      <c r="G92" s="15" t="n">
+        <v>0.000571096979138596</v>
+      </c>
+      <c r="H92" s="15" t="n">
+        <v>0.002535797727473143</v>
       </c>
     </row>
     <row r="93">
@@ -2759,25 +2759,25 @@
         </is>
       </c>
       <c r="B93" s="15" t="n">
-        <v>0.01269462804916932</v>
+        <v>0.0107415202248482</v>
       </c>
       <c r="C93" s="15" t="n">
-        <v>0.007419490803772799</v>
+        <v>0.004889809304654768</v>
       </c>
       <c r="D93" s="15" t="n">
-        <v>0.01749451716028494</v>
+        <v>0.007854528742709199</v>
       </c>
       <c r="E93" s="15" t="n">
-        <v>0.02056671642193719</v>
+        <v>1.0261733683458e-05</v>
       </c>
       <c r="F93" s="15" t="n">
-        <v>0.06400178396751266</v>
+        <v>0.005695397386688006</v>
       </c>
       <c r="G93" s="15" t="n">
-        <v>0.06400178396751266</v>
+        <v>0.005695397386688006</v>
       </c>
       <c r="H93" s="15" t="n">
-        <v>0.02562728763051969</v>
+        <v>0.006904455804449761</v>
       </c>
     </row>
     <row r="94">
@@ -2787,25 +2787,25 @@
         </is>
       </c>
       <c r="B94" s="16" t="n">
-        <v>-0.05060454568853401</v>
+        <v>-0.04752776421821448</v>
       </c>
       <c r="C94" s="16" t="n">
-        <v>-0.0965534607802202</v>
+        <v>-0.08040486919679646</v>
       </c>
       <c r="D94" s="16" t="n">
-        <v>-0.1305433417229257</v>
+        <v>-0.1036569453885952</v>
       </c>
       <c r="E94" s="16" t="n">
-        <v>-0.1808707473277017</v>
+        <v>-0.1591941916674442</v>
       </c>
       <c r="F94" s="16" t="n">
-        <v>-0.2880860673199606</v>
+        <v>-0.2624691147910039</v>
       </c>
       <c r="G94" s="16" t="n">
-        <v>-0.2880860673199606</v>
+        <v>-0.2624691147910038</v>
       </c>
       <c r="H94" s="16" t="n">
-        <v>-0.1006088589210479</v>
+        <v>-0.08981096597230198</v>
       </c>
     </row>
     <row r="95">
@@ -2815,25 +2815,25 @@
         </is>
       </c>
       <c r="B95" s="15" t="n">
-        <v>0.01113464979454659</v>
+        <v>0.01238288607362836</v>
       </c>
       <c r="C95" s="15" t="n">
-        <v>0.01281032755056466</v>
+        <v>0.01425819180947197</v>
       </c>
       <c r="D95" s="16" t="n">
-        <v>-0.01775112125413525</v>
+        <v>-0.01558433025888284</v>
       </c>
       <c r="E95" s="16" t="n">
-        <v>-0.04699598359215552</v>
+        <v>-0.04150083994203325</v>
       </c>
       <c r="F95" s="16" t="n">
-        <v>-0.1898875375619469</v>
+        <v>-0.1718035365136157</v>
       </c>
       <c r="G95" s="16" t="n">
-        <v>-0.139503053481145</v>
+        <v>-0.1202943282677335</v>
       </c>
       <c r="H95" s="16" t="n">
-        <v>-0.04144706603757154</v>
+        <v>-0.03430362448331414</v>
       </c>
     </row>
     <row r="96">
@@ -2843,10 +2843,10 @@
         </is>
       </c>
       <c r="B96" s="16" t="n">
-        <v>-0.01340277855125094</v>
+        <v>-0.002780384651533518</v>
       </c>
       <c r="C96" s="16" t="n">
-        <v>-0.01198453722536663</v>
+        <v>-0.000537321457946937</v>
       </c>
       <c r="D96" s="15" t="n">
         <v>0</v>
@@ -2858,10 +2858,10 @@
         <v>0</v>
       </c>
       <c r="G96" s="15" t="n">
-        <v>0.1289264057238508</v>
+        <v>0.07496588721849351</v>
       </c>
       <c r="H96" s="15" t="n">
-        <v>0.05084512145601305</v>
+        <v>0.03411428125857064</v>
       </c>
     </row>
     <row r="97">
@@ -2871,10 +2871,10 @@
         </is>
       </c>
       <c r="B97" s="16" t="n">
-        <v>-0.01312409980664542</v>
+        <v>-0.01889066495858382</v>
       </c>
       <c r="C97" s="16" t="n">
-        <v>-0.01013823570198658</v>
+        <v>-0.01570721874534875</v>
       </c>
       <c r="D97" s="15" t="n">
         <v>0</v>
@@ -2886,10 +2886,10 @@
         <v>0</v>
       </c>
       <c r="G97" s="16" t="n">
-        <v>-0.371558075327248</v>
+        <v>-0.3661464200943989</v>
       </c>
       <c r="H97" s="16" t="n">
-        <v>-0.1351092347622971</v>
+        <v>-0.1326168062051617</v>
       </c>
     </row>
     <row r="98">
@@ -2898,11 +2898,11 @@
           <t>2022-05</t>
         </is>
       </c>
-      <c r="B98" s="15" t="n">
-        <v>0.001314798839433528</v>
-      </c>
-      <c r="C98" s="15" t="n">
-        <v>0.001433075908586545</v>
+      <c r="B98" s="16" t="n">
+        <v>-0.008757187686515455</v>
+      </c>
+      <c r="C98" s="16" t="n">
+        <v>-0.009804300360304108</v>
       </c>
       <c r="D98" s="15" t="n">
         <v>0</v>
@@ -2914,10 +2914,10 @@
         <v>0</v>
       </c>
       <c r="G98" s="16" t="n">
-        <v>-0.1443492901581959</v>
+        <v>-0.1024694823424812</v>
       </c>
       <c r="H98" s="16" t="n">
-        <v>-0.03626588820152932</v>
+        <v>-0.02053160912828789</v>
       </c>
     </row>
     <row r="99">
@@ -2927,10 +2927,10 @@
         </is>
       </c>
       <c r="B99" s="16" t="n">
-        <v>-0.006331319723415385</v>
+        <v>-0.008292353774216887</v>
       </c>
       <c r="C99" s="16" t="n">
-        <v>-0.005900025248675944</v>
+        <v>-0.007514203447170131</v>
       </c>
       <c r="D99" s="15" t="n">
         <v>0</v>
@@ -2942,10 +2942,10 @@
         <v>0</v>
       </c>
       <c r="G99" s="16" t="n">
-        <v>-0.2503737806141946</v>
+        <v>-0.266580806180883</v>
       </c>
       <c r="H99" s="16" t="n">
-        <v>-0.08051381468674468</v>
+        <v>-0.08712982899269706</v>
       </c>
     </row>
     <row r="100">
@@ -2955,10 +2955,10 @@
         </is>
       </c>
       <c r="B100" s="15" t="n">
-        <v>0.001149794590374009</v>
-      </c>
-      <c r="C100" s="16" t="n">
-        <v>-0.000173626136668825</v>
+        <v>0.002429683518438752</v>
+      </c>
+      <c r="C100" s="15" t="n">
+        <v>0.0005135324426452921</v>
       </c>
       <c r="D100" s="15" t="n">
         <v>0</v>
@@ -2970,10 +2970,10 @@
         <v>0</v>
       </c>
       <c r="G100" s="15" t="n">
-        <v>0.3558505582749116</v>
+        <v>0.3923571931106742</v>
       </c>
       <c r="H100" s="15" t="n">
-        <v>0.1134847130975405</v>
+        <v>0.1234910031761829</v>
       </c>
     </row>
     <row r="101">
@@ -2983,10 +2983,10 @@
         </is>
       </c>
       <c r="B101" s="16" t="n">
-        <v>-0.02155059849385299</v>
+        <v>-0.01964415694485233</v>
       </c>
       <c r="C101" s="16" t="n">
-        <v>-0.01757767045784364</v>
+        <v>-0.01595564687619777</v>
       </c>
       <c r="D101" s="15" t="n">
         <v>0</v>
@@ -2998,10 +2998,10 @@
         <v>0</v>
       </c>
       <c r="G101" s="16" t="n">
-        <v>-0.1434774395279171</v>
+        <v>-0.1480088577551232</v>
       </c>
       <c r="H101" s="16" t="n">
-        <v>-0.04469085183165156</v>
+        <v>-0.0463646668952803</v>
       </c>
     </row>
     <row r="102">
@@ -3011,10 +3011,10 @@
         </is>
       </c>
       <c r="B102" s="16" t="n">
-        <v>-0.01812907008354325</v>
+        <v>-0.02399291996870989</v>
       </c>
       <c r="C102" s="16" t="n">
-        <v>-0.01607194944481971</v>
+        <v>-0.02090362747411001</v>
       </c>
       <c r="D102" s="15" t="n">
         <v>0</v>
@@ -3026,10 +3026,10 @@
         <v>0</v>
       </c>
       <c r="G102" s="16" t="n">
-        <v>-0.2934742705193119</v>
+        <v>-0.2990717411039167</v>
       </c>
       <c r="H102" s="16" t="n">
-        <v>-0.1026301600111303</v>
+        <v>-0.1049897646975497</v>
       </c>
     </row>
     <row r="103">
@@ -3039,10 +3039,10 @@
         </is>
       </c>
       <c r="B103" s="16" t="n">
-        <v>-0.01942263102407837</v>
+        <v>-0.01032560443923869</v>
       </c>
       <c r="C103" s="16" t="n">
-        <v>-0.01924321711016685</v>
+        <v>-0.01190490812420852</v>
       </c>
       <c r="D103" s="15" t="n">
         <v>0</v>
@@ -3054,10 +3054,10 @@
         <v>0</v>
       </c>
       <c r="G103" s="15" t="n">
-        <v>0.02210519773846742</v>
+        <v>0.09160116342291902</v>
       </c>
       <c r="H103" s="15" t="n">
-        <v>0.01596984198645601</v>
+        <v>0.03900766752836127</v>
       </c>
     </row>
     <row r="104">
@@ -3067,10 +3067,10 @@
         </is>
       </c>
       <c r="B104" s="15" t="n">
-        <v>0.02788928407351543</v>
+        <v>0.03027681609066057</v>
       </c>
       <c r="C104" s="15" t="n">
-        <v>0.02408228485544739</v>
+        <v>0.02630402121196851</v>
       </c>
       <c r="D104" s="15" t="n">
         <v>0</v>
@@ -3082,10 +3082,10 @@
         <v>0</v>
       </c>
       <c r="G104" s="15" t="n">
-        <v>0.1310850007701556</v>
+        <v>0.1009989080911915</v>
       </c>
       <c r="H104" s="15" t="n">
-        <v>0.05299406486415714</v>
+        <v>0.04366973442449473</v>
       </c>
     </row>
     <row r="105">
@@ -3094,11 +3094,11 @@
           <t>2022-12</t>
         </is>
       </c>
-      <c r="B105" s="16" t="n">
-        <v>-0.004572578863880738</v>
-      </c>
-      <c r="C105" s="16" t="n">
-        <v>-0.001987638192057383</v>
+      <c r="B105" s="15" t="n">
+        <v>0.009385362921058292</v>
+      </c>
+      <c r="C105" s="15" t="n">
+        <v>0.01103470878919155</v>
       </c>
       <c r="D105" s="15" t="n">
         <v>0</v>
@@ -3110,10 +3110,10 @@
         <v>0</v>
       </c>
       <c r="G105" s="16" t="n">
-        <v>-0.2534353517750249</v>
+        <v>-0.2506387147643933</v>
       </c>
       <c r="H105" s="16" t="n">
-        <v>-0.08848022062201079</v>
+        <v>-0.0873316647410185</v>
       </c>
     </row>
     <row r="106">
@@ -3123,10 +3123,10 @@
         </is>
       </c>
       <c r="B106" s="15" t="n">
-        <v>0.02232073366369258</v>
+        <v>0.02793411369777754</v>
       </c>
       <c r="C106" s="15" t="n">
-        <v>0.01845318202060331</v>
+        <v>0.02297884319308841</v>
       </c>
       <c r="D106" s="15" t="n">
         <v>0</v>
@@ -3138,10 +3138,10 @@
         <v>0</v>
       </c>
       <c r="G106" s="15" t="n">
-        <v>0.370806910763359</v>
+        <v>0.339523511638867</v>
       </c>
       <c r="H106" s="15" t="n">
-        <v>0.1152952332528665</v>
+        <v>0.1068238114307618</v>
       </c>
     </row>
     <row r="107">
@@ -3151,10 +3151,10 @@
         </is>
       </c>
       <c r="B107" s="16" t="n">
-        <v>-0.06704184153916204</v>
+        <v>-0.06432006122028966</v>
       </c>
       <c r="C107" s="16" t="n">
-        <v>-0.1030607737160563</v>
+        <v>-0.1014442987829183</v>
       </c>
       <c r="D107" s="16" t="n">
         <v>-0.1157266207586112</v>
@@ -3166,10 +3166,10 @@
         <v>-0.1157266207586114</v>
       </c>
       <c r="G107" s="16" t="n">
-        <v>-0.0999225349157431</v>
+        <v>-0.04593007062435205</v>
       </c>
       <c r="H107" s="16" t="n">
-        <v>-0.03053237081393645</v>
+        <v>-0.01113636419196873</v>
       </c>
     </row>
     <row r="108">
@@ -3179,25 +3179,25 @@
         </is>
       </c>
       <c r="B108" s="15" t="n">
-        <v>0.1127137574826453</v>
+        <v>0.1051751333031892</v>
       </c>
       <c r="C108" s="15" t="n">
-        <v>0.1815544131807121</v>
+        <v>0.1644186202497524</v>
       </c>
       <c r="D108" s="15" t="n">
-        <v>0.2240771582511149</v>
+        <v>0.1996534391125415</v>
       </c>
       <c r="E108" s="15" t="n">
-        <v>0.2240771582511149</v>
+        <v>0.1996534391125415</v>
       </c>
       <c r="F108" s="15" t="n">
-        <v>0.2240771582511149</v>
+        <v>0.1996534391125413</v>
       </c>
       <c r="G108" s="15" t="n">
-        <v>0.2240771582511148</v>
+        <v>0.1996534391125413</v>
       </c>
       <c r="H108" s="15" t="n">
-        <v>0.07403059303220871</v>
+        <v>0.06689951888555545</v>
       </c>
     </row>
     <row r="109">
@@ -3207,25 +3207,25 @@
         </is>
       </c>
       <c r="B109" s="15" t="n">
-        <v>0.002322342807406396</v>
-      </c>
-      <c r="C109" s="15" t="n">
-        <v>0.002870746225500653</v>
-      </c>
-      <c r="D109" s="15" t="n">
-        <v>0.003112227796682187</v>
+        <v>0.002969047065691343</v>
+      </c>
+      <c r="C109" s="16" t="n">
+        <v>-0.001935175157395829</v>
+      </c>
+      <c r="D109" s="16" t="n">
+        <v>-0.004914450927922531</v>
       </c>
       <c r="E109" s="16" t="n">
-        <v>-0.01455285944305651</v>
-      </c>
-      <c r="F109" s="15" t="n">
-        <v>0.003112227796682187</v>
-      </c>
-      <c r="G109" s="15" t="n">
-        <v>0.003112227796682187</v>
+        <v>-0.02243818610755621</v>
+      </c>
+      <c r="F109" s="16" t="n">
+        <v>-0.00491445092792242</v>
+      </c>
+      <c r="G109" s="16" t="n">
+        <v>-0.00491445092792242</v>
       </c>
       <c r="H109" s="15" t="n">
-        <v>0.003046067067633551</v>
+        <v>0.000382094272932675</v>
       </c>
     </row>
     <row r="110">
@@ -3235,25 +3235,25 @@
         </is>
       </c>
       <c r="B110" s="15" t="n">
-        <v>0.0450984822886551</v>
+        <v>0.03977944455312388</v>
       </c>
       <c r="C110" s="15" t="n">
-        <v>0.08746596486721024</v>
+        <v>0.08316140959853759</v>
       </c>
       <c r="D110" s="15" t="n">
-        <v>0.1279048025985219</v>
+        <v>0.1239972063106549</v>
       </c>
       <c r="E110" s="15" t="n">
-        <v>0.1112522478945826</v>
+        <v>0.1074023439410285</v>
       </c>
       <c r="F110" s="15" t="n">
-        <v>0.1794282128270799</v>
+        <v>0.1753421150503607</v>
       </c>
       <c r="G110" s="15" t="n">
-        <v>0.1794282128270797</v>
+        <v>0.1753421150503602</v>
       </c>
       <c r="H110" s="15" t="n">
-        <v>0.05917580636416897</v>
+        <v>0.0579646930220068</v>
       </c>
     </row>
     <row r="111">
@@ -3263,25 +3263,25 @@
         </is>
       </c>
       <c r="B111" s="15" t="n">
-        <v>0.05148113601970139</v>
+        <v>0.07077701812872617</v>
       </c>
       <c r="C111" s="15" t="n">
-        <v>0.1096904918544501</v>
+        <v>0.1419969294799481</v>
       </c>
       <c r="D111" s="15" t="n">
-        <v>0.1585036029876836</v>
+        <v>0.2029825025661567</v>
       </c>
       <c r="E111" s="15" t="n">
-        <v>0.1367619198433947</v>
+        <v>0.1603089982200752</v>
       </c>
       <c r="F111" s="15" t="n">
-        <v>0.1585036029876841</v>
+        <v>0.2029825025661572</v>
       </c>
       <c r="G111" s="15" t="n">
-        <v>0.1585036029876836</v>
+        <v>0.2029825025661569</v>
       </c>
       <c r="H111" s="15" t="n">
-        <v>0.05243420175791935</v>
+        <v>0.06591501854521198</v>
       </c>
     </row>
     <row r="112">
@@ -3291,25 +3291,25 @@
         </is>
       </c>
       <c r="B112" s="15" t="n">
-        <v>0.04676021492702476</v>
+        <v>0.04825255363454839</v>
       </c>
       <c r="C112" s="15" t="n">
-        <v>0.08895264340433663</v>
+        <v>0.0938253564983369</v>
       </c>
       <c r="D112" s="15" t="n">
-        <v>0.1136721419234177</v>
+        <v>0.1206248216542256</v>
       </c>
       <c r="E112" s="15" t="n">
-        <v>0.1100079053123322</v>
+        <v>0.1167120484535942</v>
       </c>
       <c r="F112" s="15" t="n">
-        <v>0.1136721419234174</v>
+        <v>0.1206248216542252</v>
       </c>
       <c r="G112" s="15" t="n">
-        <v>0.1136721419234181</v>
+        <v>0.120624821654226</v>
       </c>
       <c r="H112" s="15" t="n">
-        <v>0.03830490179364787</v>
+        <v>0.04047743332839904</v>
       </c>
     </row>
     <row r="113">
@@ -3319,25 +3319,25 @@
         </is>
       </c>
       <c r="B113" s="16" t="n">
-        <v>-0.04159509189440403</v>
+        <v>-0.05253822259860098</v>
       </c>
       <c r="C113" s="16" t="n">
-        <v>-0.08654311888855004</v>
+        <v>-0.09806447500905124</v>
       </c>
       <c r="D113" s="16" t="n">
-        <v>-0.1086850035666471</v>
+        <v>-0.1202919463419843</v>
       </c>
       <c r="E113" s="16" t="n">
-        <v>-0.0636553228114124</v>
+        <v>-0.07545159307137594</v>
       </c>
       <c r="F113" s="16" t="n">
-        <v>-0.05959500753555479</v>
+        <v>-0.07184121339639427</v>
       </c>
       <c r="G113" s="16" t="n">
-        <v>-0.05959500753555479</v>
+        <v>-0.07184121339639438</v>
       </c>
       <c r="H113" s="16" t="n">
-        <v>-0.01742803104782731</v>
+        <v>-0.02168195881860746</v>
       </c>
     </row>
     <row r="114">
@@ -3347,25 +3347,25 @@
         </is>
       </c>
       <c r="B114" s="16" t="n">
-        <v>-0.05045636554347976</v>
+        <v>-0.05212707458160281</v>
       </c>
       <c r="C114" s="16" t="n">
-        <v>-0.06294235246472835</v>
+        <v>-0.06384645355920515</v>
       </c>
       <c r="D114" s="16" t="n">
-        <v>-0.07862569776136241</v>
+        <v>-0.07897416124054268</v>
       </c>
       <c r="E114" s="16" t="n">
-        <v>-0.1041024079691298</v>
+        <v>-0.1047261691571125</v>
       </c>
       <c r="F114" s="16" t="n">
-        <v>-0.1686685353618833</v>
+        <v>-0.1692584615215289</v>
       </c>
       <c r="G114" s="16" t="n">
-        <v>-0.1686685353618834</v>
+        <v>-0.1692584615215292</v>
       </c>
       <c r="H114" s="16" t="n">
-        <v>-0.05790338400340812</v>
+        <v>-0.05811550932801845</v>
       </c>
     </row>
     <row r="115">
@@ -3375,25 +3375,25 @@
         </is>
       </c>
       <c r="B115" s="16" t="n">
-        <v>-0.01407015526271371</v>
+        <v>-0.01765460037580957</v>
       </c>
       <c r="C115" s="16" t="n">
-        <v>-0.05073143451973438</v>
+        <v>-0.05130103077915749</v>
       </c>
       <c r="D115" s="16" t="n">
-        <v>-0.1015944638148456</v>
+        <v>-0.09655190017960312</v>
       </c>
       <c r="E115" s="16" t="n">
-        <v>-0.1245239435123004</v>
+        <v>-0.1184520201991199</v>
       </c>
       <c r="F115" s="16" t="n">
-        <v>-0.108294443914957</v>
+        <v>-0.09042592316459183</v>
       </c>
       <c r="G115" s="16" t="n">
-        <v>-0.1082944439149578</v>
+        <v>-0.09042592316459253</v>
       </c>
       <c r="H115" s="16" t="n">
-        <v>-0.03430547063525213</v>
+        <v>-0.02784410010679195</v>
       </c>
     </row>
     <row r="116">
@@ -3403,25 +3403,25 @@
         </is>
       </c>
       <c r="B116" s="15" t="n">
-        <v>0.05954061049065928</v>
+        <v>0.06355566977697169</v>
       </c>
       <c r="C116" s="15" t="n">
-        <v>0.08407695886261844</v>
+        <v>0.08907652234311826</v>
       </c>
       <c r="D116" s="15" t="n">
-        <v>0.1172623675846158</v>
+        <v>0.1264230081956648</v>
       </c>
       <c r="E116" s="15" t="n">
-        <v>0.1189019141089995</v>
+        <v>0.1347984584197461</v>
       </c>
       <c r="F116" s="15" t="n">
-        <v>0.2842741321082856</v>
+        <v>0.3472574420278935</v>
       </c>
       <c r="G116" s="15" t="n">
-        <v>0.2842741321082858</v>
+        <v>0.3472574420278938</v>
       </c>
       <c r="H116" s="15" t="n">
-        <v>0.08917449753998996</v>
+        <v>0.1069919686435905</v>
       </c>
     </row>
     <row r="117">
@@ -3431,25 +3431,25 @@
         </is>
       </c>
       <c r="B117" s="15" t="n">
-        <v>0.05297246727446581</v>
+        <v>0.06675487811066882</v>
       </c>
       <c r="C117" s="15" t="n">
-        <v>0.09726791906319621</v>
+        <v>0.1126853249070437</v>
       </c>
       <c r="D117" s="15" t="n">
-        <v>0.1314030207536361</v>
+        <v>0.1478031208157358</v>
       </c>
       <c r="E117" s="15" t="n">
-        <v>0.1251843561259936</v>
+        <v>0.1392284191793765</v>
       </c>
       <c r="F117" s="15" t="n">
-        <v>0.151006013044112</v>
+        <v>0.1700957947405011</v>
       </c>
       <c r="G117" s="15" t="n">
-        <v>0.151006013044112</v>
+        <v>0.1700957947405011</v>
       </c>
       <c r="H117" s="15" t="n">
-        <v>0.04937559183282825</v>
+        <v>0.05518893268227432</v>
       </c>
     </row>
     <row r="118">
@@ -3459,25 +3459,25 @@
         </is>
       </c>
       <c r="B118" s="15" t="n">
-        <v>0.02115472905105098</v>
+        <v>0.004136041944944102</v>
       </c>
       <c r="C118" s="15" t="n">
-        <v>0.04740397409977981</v>
+        <v>0.01317538518677397</v>
       </c>
       <c r="D118" s="15" t="n">
-        <v>0.06717619318980361</v>
+        <v>0.02140035205320401</v>
       </c>
       <c r="E118" s="15" t="n">
-        <v>0.06851202221037589</v>
+        <v>0.02411480823298007</v>
       </c>
       <c r="F118" s="15" t="n">
-        <v>0.07604178231829151</v>
+        <v>0.02323088512068439</v>
       </c>
       <c r="G118" s="15" t="n">
-        <v>0.07604178231829195</v>
+        <v>0.02323088512068461</v>
       </c>
       <c r="H118" s="15" t="n">
-        <v>0.0269586172200158</v>
+        <v>0.01016964898043926</v>
       </c>
     </row>
     <row r="119">
@@ -3487,25 +3487,25 @@
         </is>
       </c>
       <c r="B119" s="15" t="n">
-        <v>0.03573312749474633</v>
+        <v>0.05171541977024763</v>
       </c>
       <c r="C119" s="15" t="n">
-        <v>0.08268105356462009</v>
+        <v>0.1070622544493802</v>
       </c>
       <c r="D119" s="15" t="n">
-        <v>0.1236572244115215</v>
+        <v>0.1620209006306683</v>
       </c>
       <c r="E119" s="15" t="n">
-        <v>0.1296915043000881</v>
+        <v>0.1701588517542334</v>
       </c>
       <c r="F119" s="15" t="n">
-        <v>0.1413195278097543</v>
+        <v>0.1859044304179649</v>
       </c>
       <c r="G119" s="15" t="n">
-        <v>0.1413195278097545</v>
+        <v>0.1859044304179653</v>
       </c>
       <c r="H119" s="15" t="n">
-        <v>0.04753921392185356</v>
+        <v>0.06119160898679077</v>
       </c>
     </row>
     <row r="120">
@@ -3515,25 +3515,25 @@
         </is>
       </c>
       <c r="B120" s="15" t="n">
-        <v>0.01033156664365875</v>
-      </c>
-      <c r="C120" s="16" t="n">
-        <v>-0.006517830467199892</v>
-      </c>
-      <c r="D120" s="16" t="n">
-        <v>-0.01989607529727766</v>
-      </c>
-      <c r="E120" s="16" t="n">
-        <v>-0.02908296306283775</v>
+        <v>0.02966339077526392</v>
+      </c>
+      <c r="C120" s="15" t="n">
+        <v>0.01854703766940346</v>
+      </c>
+      <c r="D120" s="15" t="n">
+        <v>0.009302151256766368</v>
+      </c>
+      <c r="E120" s="15" t="n">
+        <v>0.001264680496255277</v>
       </c>
       <c r="F120" s="15" t="n">
-        <v>0.01457350775485877</v>
+        <v>0.04915646034839694</v>
       </c>
       <c r="G120" s="15" t="n">
-        <v>0.01457350775485855</v>
+        <v>0.04915646034839671</v>
       </c>
       <c r="H120" s="15" t="n">
-        <v>0.006422114520268307</v>
+        <v>0.01786859743638325</v>
       </c>
     </row>
     <row r="121">
@@ -3543,25 +3543,25 @@
         </is>
       </c>
       <c r="B121" s="16" t="n">
-        <v>-0.02035634560463573</v>
+        <v>-0.0200945700206161</v>
       </c>
       <c r="C121" s="16" t="n">
-        <v>-0.03308432862204624</v>
+        <v>-0.03170582642138753</v>
       </c>
       <c r="D121" s="16" t="n">
-        <v>-0.05910155384283011</v>
+        <v>-0.05753190683091203</v>
       </c>
       <c r="E121" s="16" t="n">
-        <v>-0.04072273766279055</v>
+        <v>-0.03981699246983583</v>
       </c>
       <c r="F121" s="16" t="n">
-        <v>-0.1383297726598313</v>
+        <v>-0.1356178223997505</v>
       </c>
       <c r="G121" s="16" t="n">
-        <v>-0.1383297726598309</v>
+        <v>-0.1356178223997503</v>
       </c>
       <c r="H121" s="16" t="n">
-        <v>-0.0450702826158399</v>
+        <v>-0.04405759714657852</v>
       </c>
     </row>
     <row r="122">
@@ -3571,25 +3571,25 @@
         </is>
       </c>
       <c r="B122" s="15" t="n">
-        <v>0.02608254473003013</v>
+        <v>0.02884193492055531</v>
       </c>
       <c r="C122" s="15" t="n">
-        <v>0.0343994697761445</v>
+        <v>0.03730730922141712</v>
       </c>
       <c r="D122" s="15" t="n">
-        <v>0.05902944647122466</v>
+        <v>0.05662137159968883</v>
       </c>
       <c r="E122" s="15" t="n">
-        <v>0.06266078689454835</v>
+        <v>0.05945293932955975</v>
       </c>
       <c r="F122" s="15" t="n">
-        <v>0.2272781331945692</v>
+        <v>0.2149288767504793</v>
       </c>
       <c r="G122" s="15" t="n">
-        <v>0.2272781331945692</v>
+        <v>0.2149288767504791</v>
       </c>
       <c r="H122" s="15" t="n">
-        <v>0.07238092186664202</v>
+        <v>0.06879624349054803</v>
       </c>
     </row>
     <row r="123">
@@ -3599,25 +3599,25 @@
         </is>
       </c>
       <c r="B123" s="15" t="n">
-        <v>0.04818085774617398</v>
+        <v>0.05851324763314403</v>
       </c>
       <c r="C123" s="15" t="n">
-        <v>0.1041553580686365</v>
+        <v>0.1159580804653128</v>
       </c>
       <c r="D123" s="15" t="n">
-        <v>0.1409149468996029</v>
+        <v>0.1538755988480673</v>
       </c>
       <c r="E123" s="15" t="n">
-        <v>0.160139615688141</v>
+        <v>0.1790269250374465</v>
       </c>
       <c r="F123" s="15" t="n">
-        <v>0.164988953537027</v>
+        <v>0.1845072855934988</v>
       </c>
       <c r="G123" s="15" t="n">
-        <v>0.164988953537027</v>
+        <v>0.1845072855934988</v>
       </c>
       <c r="H123" s="15" t="n">
-        <v>0.05371367384923365</v>
+        <v>0.05961033246852065</v>
       </c>
     </row>
     <row r="124">
@@ -3626,26 +3626,26 @@
           <t>2024-07</t>
         </is>
       </c>
-      <c r="B124" s="16" t="n">
-        <v>-0.003276270752297305</v>
+      <c r="B124" s="15" t="n">
+        <v>0.002023596883886647</v>
       </c>
       <c r="C124" s="16" t="n">
-        <v>-0.02939837874448237</v>
+        <v>-0.01259122048373185</v>
       </c>
       <c r="D124" s="16" t="n">
-        <v>-0.07288633073808259</v>
+        <v>-0.05022954579430272</v>
       </c>
       <c r="E124" s="16" t="n">
-        <v>-0.08218997655446891</v>
+        <v>-0.06008568581202455</v>
       </c>
       <c r="F124" s="16" t="n">
-        <v>-0.05967286887070743</v>
+        <v>-0.03636707971130648</v>
       </c>
       <c r="G124" s="16" t="n">
-        <v>-0.05967286887070733</v>
+        <v>-0.03636707971130626</v>
       </c>
       <c r="H124" s="16" t="n">
-        <v>-0.01565499647047342</v>
+        <v>-0.007511544933297865</v>
       </c>
     </row>
     <row r="125">
@@ -3655,25 +3655,25 @@
         </is>
       </c>
       <c r="B125" s="15" t="n">
-        <v>0.005110466119120805</v>
+        <v>0.001482515317250188</v>
       </c>
       <c r="C125" s="15" t="n">
-        <v>0.007518842947401794</v>
+        <v>0.004571604305015464</v>
       </c>
       <c r="D125" s="16" t="n">
-        <v>-0.01582171256328657</v>
-      </c>
-      <c r="E125" s="15" t="n">
-        <v>0.01405760286681246</v>
+        <v>-0.039631970673079</v>
+      </c>
+      <c r="E125" s="16" t="n">
+        <v>-0.02623818073776885</v>
       </c>
       <c r="F125" s="15" t="n">
-        <v>0.07612106589690981</v>
+        <v>0.001746911625613023</v>
       </c>
       <c r="G125" s="15" t="n">
-        <v>0.07612106589690937</v>
+        <v>0.001746911625612579</v>
       </c>
       <c r="H125" s="15" t="n">
-        <v>0.03021194640028502</v>
+        <v>0.00648992280787275</v>
       </c>
     </row>
     <row r="126">
@@ -3683,25 +3683,25 @@
         </is>
       </c>
       <c r="B126" s="15" t="n">
-        <v>0.03153132216914467</v>
+        <v>0.01252254204228076</v>
       </c>
       <c r="C126" s="15" t="n">
-        <v>0.04063785580511947</v>
-      </c>
-      <c r="D126" s="15" t="n">
-        <v>0.03426889045825599</v>
+        <v>0.001681102467018469</v>
+      </c>
+      <c r="D126" s="16" t="n">
+        <v>-0.02936818545736064</v>
       </c>
       <c r="E126" s="15" t="n">
-        <v>0.08014589892266709</v>
+        <v>0.03633899079439917</v>
       </c>
       <c r="F126" s="15" t="n">
-        <v>0.187110283467593</v>
+        <v>0.07099966314186101</v>
       </c>
       <c r="G126" s="15" t="n">
-        <v>0.187110283467593</v>
+        <v>0.07099966314186101</v>
       </c>
       <c r="H126" s="15" t="n">
-        <v>0.06144086486723066</v>
+        <v>0.02684661883462058</v>
       </c>
     </row>
     <row r="127">
@@ -3711,25 +3711,25 @@
         </is>
       </c>
       <c r="B127" s="16" t="n">
-        <v>-0.01330120432968218</v>
+        <v>-0.01351454325571311</v>
       </c>
       <c r="C127" s="16" t="n">
-        <v>-0.02870456929556864</v>
+        <v>-0.03491442095175401</v>
       </c>
       <c r="D127" s="16" t="n">
-        <v>-0.02807690085958114</v>
+        <v>-0.04273316852217701</v>
       </c>
       <c r="E127" s="16" t="n">
-        <v>-0.00726733541629665</v>
-      </c>
-      <c r="F127" s="15" t="n">
-        <v>0.02415333787551765</v>
-      </c>
-      <c r="G127" s="15" t="n">
-        <v>0.02415333787551788</v>
-      </c>
-      <c r="H127" s="15" t="n">
-        <v>0.01031754928842687</v>
+        <v>-0.03549192754100472</v>
+      </c>
+      <c r="F127" s="16" t="n">
+        <v>-0.02297745450399102</v>
+      </c>
+      <c r="G127" s="16" t="n">
+        <v>-0.0229774545039908</v>
+      </c>
+      <c r="H127" s="16" t="n">
+        <v>-0.005168984162214452</v>
       </c>
     </row>
     <row r="128">
@@ -3739,25 +3739,25 @@
         </is>
       </c>
       <c r="B128" s="15" t="n">
-        <v>0.02849135566573446</v>
+        <v>0.03508590885950192</v>
       </c>
       <c r="C128" s="15" t="n">
-        <v>0.04256632282033035</v>
+        <v>0.05568647828771756</v>
       </c>
       <c r="D128" s="15" t="n">
-        <v>0.09403807179228264</v>
+        <v>0.1202591598579885</v>
       </c>
       <c r="E128" s="15" t="n">
-        <v>0.05096077486950335</v>
+        <v>0.06488452348318652</v>
       </c>
       <c r="F128" s="15" t="n">
-        <v>0.1615575755045267</v>
+        <v>0.1893969206479695</v>
       </c>
       <c r="G128" s="15" t="n">
-        <v>0.1615575755045267</v>
+        <v>0.1893969206479693</v>
       </c>
       <c r="H128" s="15" t="n">
-        <v>0.05363236265235982</v>
+        <v>0.06206190647809318</v>
       </c>
     </row>
     <row r="129">
@@ -3767,25 +3767,25 @@
         </is>
       </c>
       <c r="B129" s="16" t="n">
-        <v>-0.03038225785992099</v>
+        <v>-0.0228071093487201</v>
       </c>
       <c r="C129" s="16" t="n">
-        <v>-0.04942525810621179</v>
+        <v>-0.0298970722567915</v>
       </c>
       <c r="D129" s="16" t="n">
-        <v>-0.06263850752044808</v>
+        <v>-0.03548647884703315</v>
       </c>
       <c r="E129" s="16" t="n">
-        <v>-0.08369065164326983</v>
-      </c>
-      <c r="F129" s="16" t="n">
-        <v>-0.02392822893758195</v>
-      </c>
-      <c r="G129" s="16" t="n">
-        <v>-0.02392822893758173</v>
-      </c>
-      <c r="H129" s="16" t="n">
-        <v>-0.004801092561094622</v>
+        <v>-0.07055650447923689</v>
+      </c>
+      <c r="F129" s="15" t="n">
+        <v>0.004345098831721294</v>
+      </c>
+      <c r="G129" s="15" t="n">
+        <v>0.004345098831721516</v>
+      </c>
+      <c r="H129" s="15" t="n">
+        <v>0.0048193527792455</v>
       </c>
     </row>
     <row r="130">
@@ -3795,25 +3795,25 @@
         </is>
       </c>
       <c r="B130" s="15" t="n">
-        <v>0.01622974243341169</v>
+        <v>0.01886237215422825</v>
       </c>
       <c r="C130" s="16" t="n">
-        <v>-0.01019897464454067</v>
+        <v>-0.008981655051958026</v>
       </c>
       <c r="D130" s="16" t="n">
-        <v>-0.008706472831536471</v>
+        <v>-0.01127809447877726</v>
       </c>
       <c r="E130" s="16" t="n">
-        <v>-0.02178293241755025</v>
+        <v>-0.02452604907667888</v>
       </c>
       <c r="F130" s="15" t="n">
-        <v>0.04269269546317367</v>
+        <v>0.03779753055951907</v>
       </c>
       <c r="G130" s="15" t="n">
-        <v>0.04269269546317389</v>
+        <v>0.03779753055951929</v>
       </c>
       <c r="H130" s="15" t="n">
-        <v>0.01797905622541229</v>
+        <v>0.01639758943045511</v>
       </c>
     </row>
     <row r="131">
@@ -3823,25 +3823,25 @@
         </is>
       </c>
       <c r="B131" s="16" t="n">
-        <v>-0.006498344922988175</v>
+        <v>-0.01214361608828374</v>
       </c>
       <c r="C131" s="16" t="n">
-        <v>-0.03067281053301885</v>
+        <v>-0.04724185864380659</v>
       </c>
       <c r="D131" s="16" t="n">
-        <v>-0.04897934291562911</v>
+        <v>-0.07455858091749135</v>
       </c>
       <c r="E131" s="16" t="n">
-        <v>-0.04667093560961188</v>
+        <v>-0.06592736399640553</v>
       </c>
       <c r="F131" s="16" t="n">
-        <v>-0.08992018300748918</v>
+        <v>-0.1227070541250224</v>
       </c>
       <c r="G131" s="16" t="n">
-        <v>-0.08992018300748959</v>
+        <v>-0.122707054125023</v>
       </c>
       <c r="H131" s="16" t="n">
-        <v>-0.02808801246972914</v>
+        <v>-0.03974844289359336</v>
       </c>
     </row>
     <row r="132">
@@ -3851,25 +3851,25 @@
         </is>
       </c>
       <c r="B132" s="15" t="n">
-        <v>0.02011624972026871</v>
+        <v>0.0214094778539109</v>
       </c>
       <c r="C132" s="15" t="n">
-        <v>0.02255909453455662</v>
+        <v>0.02171113494762245</v>
       </c>
       <c r="D132" s="16" t="n">
-        <v>-0.01370908890015898</v>
+        <v>-0.03380748124290922</v>
       </c>
       <c r="E132" s="16" t="n">
-        <v>-0.04219262394175205</v>
+        <v>-0.06084784433724688</v>
       </c>
       <c r="F132" s="16" t="n">
-        <v>-0.1783681154053048</v>
+        <v>-0.2434068432968929</v>
       </c>
       <c r="G132" s="16" t="n">
-        <v>-0.178368115405305</v>
+        <v>-0.243406843296893</v>
       </c>
       <c r="H132" s="16" t="n">
-        <v>-0.05726918478468535</v>
+        <v>-0.0821333525116098</v>
       </c>
     </row>
     <row r="133">
@@ -3879,25 +3879,25 @@
         </is>
       </c>
       <c r="B133" s="15" t="n">
-        <v>0.01324209148019095</v>
+        <v>0.01559605090575134</v>
       </c>
       <c r="C133" s="15" t="n">
-        <v>0.01726641464695877</v>
+        <v>0.01911811052843904</v>
       </c>
       <c r="D133" s="16" t="n">
-        <v>-0.01632463239370541</v>
+        <v>-0.01503058922433043</v>
       </c>
       <c r="E133" s="16" t="n">
-        <v>-0.0786106068088247</v>
+        <v>-0.07269736994936848</v>
       </c>
       <c r="F133" s="16" t="n">
-        <v>-0.3027410406222249</v>
+        <v>-0.2845545577816588</v>
       </c>
       <c r="G133" s="16" t="n">
-        <v>-0.07704410771515313</v>
-      </c>
-      <c r="H133" s="16" t="n">
-        <v>-0.000203484441611001</v>
+        <v>-0.05297081145716465</v>
+      </c>
+      <c r="H133" s="15" t="n">
+        <v>0.008500394479722617</v>
       </c>
     </row>
     <row r="134">
@@ -3906,11 +3906,11 @@
           <t>2025-05</t>
         </is>
       </c>
-      <c r="B134" s="15" t="n">
-        <v>0.004886804747352702</v>
-      </c>
-      <c r="C134" s="15" t="n">
-        <v>0.003917964381703553</v>
+      <c r="B134" s="16" t="n">
+        <v>-0.00563015691788038</v>
+      </c>
+      <c r="C134" s="16" t="n">
+        <v>-0.006216466388790032</v>
       </c>
       <c r="D134" s="15" t="n">
         <v>0.001421239525864148</v>
@@ -3922,10 +3922,10 @@
         <v>0.01288859829923616</v>
       </c>
       <c r="G134" s="15" t="n">
-        <v>0.2432151082000313</v>
+        <v>0.2996956932683993</v>
       </c>
       <c r="H134" s="15" t="n">
-        <v>0.07921912231267703</v>
+        <v>0.09557475679331916</v>
       </c>
     </row>
     <row r="135">
@@ -3935,25 +3935,25 @@
         </is>
       </c>
       <c r="B135" s="15" t="n">
-        <v>0.05979006507481843</v>
+        <v>0.07431058068307284</v>
       </c>
       <c r="C135" s="15" t="n">
-        <v>0.1340893792224656</v>
+        <v>0.1547626790440761</v>
       </c>
       <c r="D135" s="15" t="n">
-        <v>0.1808024665875498</v>
+        <v>0.2046404114382004</v>
       </c>
       <c r="E135" s="15" t="n">
-        <v>0.1808024665875501</v>
+        <v>0.2046404114382005</v>
       </c>
       <c r="F135" s="15" t="n">
-        <v>0.1808024665875501</v>
+        <v>0.2046404114382005</v>
       </c>
       <c r="G135" s="15" t="n">
-        <v>0.1808024665875503</v>
+        <v>0.2046404114382008</v>
       </c>
       <c r="H135" s="15" t="n">
-        <v>0.0585742334516417</v>
+        <v>0.06570974581683497</v>
       </c>
     </row>
     <row r="136">
@@ -3963,25 +3963,25 @@
         </is>
       </c>
       <c r="B136" s="15" t="n">
-        <v>0.04501340311817326</v>
+        <v>0.03904793623347591</v>
       </c>
       <c r="C136" s="15" t="n">
-        <v>0.1039373555175724</v>
+        <v>0.08490463642041401</v>
       </c>
       <c r="D136" s="15" t="n">
-        <v>0.1401927025721303</v>
+        <v>0.1121372832146976</v>
       </c>
       <c r="E136" s="15" t="n">
-        <v>0.1401927025721297</v>
+        <v>0.112137283214697</v>
       </c>
       <c r="F136" s="15" t="n">
-        <v>0.1401927025721295</v>
+        <v>0.1121372832146965</v>
       </c>
       <c r="G136" s="15" t="n">
-        <v>0.1401927025721295</v>
+        <v>0.1121372832146967</v>
       </c>
       <c r="H136" s="15" t="n">
-        <v>0.04551618928293832</v>
+        <v>0.03695280853886485</v>
       </c>
     </row>
     <row r="137">
@@ -3991,25 +3991,25 @@
         </is>
       </c>
       <c r="B137" s="15" t="n">
-        <v>0.05473732989984903</v>
+        <v>0.03537798161050909</v>
       </c>
       <c r="C137" s="15" t="n">
-        <v>0.09624610856560543</v>
+        <v>0.04196596434885813</v>
       </c>
       <c r="D137" s="15" t="n">
-        <v>0.1152640807517828</v>
+        <v>0.0404108750757084</v>
       </c>
       <c r="E137" s="15" t="n">
-        <v>0.0956937780844158</v>
+        <v>0.0221540728751688</v>
       </c>
       <c r="F137" s="15" t="n">
-        <v>0.1152640807517822</v>
+        <v>0.04041087507570751</v>
       </c>
       <c r="G137" s="15" t="n">
-        <v>0.1152640807517828</v>
+        <v>0.04041087507570817</v>
       </c>
       <c r="H137" s="15" t="n">
-        <v>0.03900313888371065</v>
+        <v>0.01577002548569562</v>
       </c>
     </row>
     <row r="138">
@@ -4019,25 +4019,25 @@
         </is>
       </c>
       <c r="B138" s="15" t="n">
-        <v>0.08686917787144033</v>
+        <v>0.08192963958456347</v>
       </c>
       <c r="C138" s="15" t="n">
-        <v>0.1204320379052451</v>
+        <v>0.1063990571834419</v>
       </c>
       <c r="D138" s="15" t="n">
-        <v>0.1537336495855628</v>
+        <v>0.1253149440594126</v>
       </c>
       <c r="E138" s="15" t="n">
-        <v>0.1188026144186862</v>
+        <v>0.1015826284197863</v>
       </c>
       <c r="F138" s="15" t="n">
-        <v>0.2039375419255592</v>
+        <v>0.174282216809446</v>
       </c>
       <c r="G138" s="15" t="n">
-        <v>0.2039375419255589</v>
+        <v>0.1742822168094456</v>
       </c>
       <c r="H138" s="15" t="n">
-        <v>0.06486855506903022</v>
+        <v>0.05613740689554225</v>
       </c>
     </row>
     <row r="139">
@@ -4047,25 +4047,25 @@
         </is>
       </c>
       <c r="B139" s="15" t="n">
-        <v>0.04088293183661262</v>
+        <v>0.04836479554048356</v>
       </c>
       <c r="C139" s="15" t="n">
-        <v>0.06074439627543127</v>
+        <v>0.07123005986374586</v>
       </c>
       <c r="D139" s="15" t="n">
-        <v>0.08698371523308035</v>
+        <v>0.09941891513153278</v>
       </c>
       <c r="E139" s="15" t="n">
-        <v>0.07681447187209289</v>
+        <v>0.08394271948323473</v>
       </c>
       <c r="F139" s="15" t="n">
-        <v>0.1208819726478125</v>
+        <v>0.1349636203590139</v>
       </c>
       <c r="G139" s="15" t="n">
-        <v>0.1208819726478125</v>
+        <v>0.1349636203590139</v>
       </c>
       <c r="H139" s="15" t="n">
-        <v>0.04261893893915891</v>
+        <v>0.04699694231776186</v>
       </c>
     </row>
     <row r="140">
@@ -4075,25 +4075,25 @@
         </is>
       </c>
       <c r="B140" s="16" t="n">
-        <v>-0.02744662502377748</v>
+        <v>-0.02161917089853782</v>
       </c>
       <c r="C140" s="16" t="n">
-        <v>-0.08349061592858288</v>
+        <v>-0.07420076129851572</v>
       </c>
       <c r="D140" s="16" t="n">
-        <v>-0.1264798483715336</v>
+        <v>-0.1153153654567373</v>
       </c>
       <c r="E140" s="16" t="n">
-        <v>-0.1214862525769564</v>
+        <v>-0.1106982738527593</v>
       </c>
       <c r="F140" s="16" t="n">
-        <v>-0.06851337987029693</v>
+        <v>-0.055617043753995</v>
       </c>
       <c r="G140" s="16" t="n">
-        <v>-0.0685133798702966</v>
+        <v>-0.05561704375399468</v>
       </c>
       <c r="H140" s="16" t="n">
-        <v>-0.01967848735640965</v>
+        <v>-0.01514318549655147</v>
       </c>
     </row>
     <row r="141">
@@ -4103,25 +4103,25 @@
         </is>
       </c>
       <c r="B141" s="16" t="n">
-        <v>-0.001766765741778142</v>
+        <v>-0.00354433052031744</v>
       </c>
       <c r="C141" s="16" t="n">
-        <v>-0.01743762222009715</v>
+        <v>-0.02003305310419701</v>
       </c>
       <c r="D141" s="16" t="n">
-        <v>-0.02562024858656187</v>
+        <v>-0.03016021812315839</v>
       </c>
       <c r="E141" s="16" t="n">
-        <v>-0.01705725098748889</v>
+        <v>-0.02485235631947202</v>
       </c>
       <c r="F141" s="16" t="n">
-        <v>-0.008832411417259323</v>
+        <v>-0.02029025037949361</v>
       </c>
       <c r="G141" s="16" t="n">
-        <v>-0.008832411417259434</v>
+        <v>-0.02029025037949361</v>
       </c>
       <c r="H141" s="16" t="n">
-        <v>-0.001457716284206323</v>
+        <v>-0.005294053873229787</v>
       </c>
     </row>
     <row r="142">
@@ -4131,25 +4131,25 @@
         </is>
       </c>
       <c r="B142" s="15" t="n">
-        <v>0.03479861402114981</v>
+        <v>0.03318224475898002</v>
       </c>
       <c r="C142" s="15" t="n">
-        <v>0.02824167388843812</v>
+        <v>0.02706073591448588</v>
       </c>
       <c r="D142" s="15" t="n">
-        <v>0.02188295834175236</v>
+        <v>0.02113175404862622</v>
       </c>
       <c r="E142" s="15" t="n">
-        <v>0.02460046035495655</v>
+        <v>0.02372445330678508</v>
       </c>
       <c r="F142" s="15" t="n">
-        <v>0.02460046035495678</v>
+        <v>0.0237244533067853</v>
       </c>
       <c r="G142" s="15" t="n">
-        <v>0.02460046035495678</v>
+        <v>0.0237244533067853</v>
       </c>
       <c r="H142" s="15" t="n">
-        <v>0.00973459487689099</v>
+        <v>0.009458315570577414</v>
       </c>
     </row>
     <row r="143">
@@ -4159,25 +4159,25 @@
         </is>
       </c>
       <c r="B143" s="15" t="n">
-        <v>0.01203343933295886</v>
+        <v>0.01010407444899419</v>
       </c>
       <c r="C143" s="16" t="n">
-        <v>-0.05290454997268201</v>
+        <v>-0.04542526094247867</v>
       </c>
       <c r="D143" s="16" t="n">
-        <v>-0.1058659388680251</v>
+        <v>-0.09308439113318168</v>
       </c>
       <c r="E143" s="16" t="n">
-        <v>-0.1135711395657558</v>
+        <v>-0.09883374050230842</v>
       </c>
       <c r="F143" s="16" t="n">
-        <v>-0.1200932115157937</v>
+        <v>-0.1054642457190624</v>
       </c>
       <c r="G143" s="16" t="n">
-        <v>-0.1200932115157937</v>
+        <v>-0.1054642457190623</v>
       </c>
       <c r="H143" s="16" t="n">
-        <v>-0.03916133241053177</v>
+        <v>-0.03382556700330619</v>
       </c>
     </row>
     <row r="144">
@@ -4187,25 +4187,25 @@
         </is>
       </c>
       <c r="B144" s="16" t="n">
-        <v>-0.08220595726419988</v>
+        <v>-0.07845687521445621</v>
       </c>
       <c r="C144" s="16" t="n">
-        <v>-0.07169613472829472</v>
+        <v>-0.06676742193858798</v>
       </c>
       <c r="D144" s="16" t="n">
-        <v>-0.04691953887245336</v>
+        <v>-0.04096163768438366</v>
       </c>
       <c r="E144" s="16" t="n">
-        <v>-0.08598895348493663</v>
+        <v>-0.08125817834443616</v>
       </c>
       <c r="F144" s="16" t="n">
-        <v>-0.174279629450085</v>
+        <v>-0.1654946221868014</v>
       </c>
       <c r="G144" s="16" t="n">
-        <v>-0.1742796294500849</v>
+        <v>-0.1654946221868014</v>
       </c>
       <c r="H144" s="16" t="n">
-        <v>-0.05893830872014871</v>
+        <v>-0.05559022116255175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>